<commit_message>
Archive qualified DMC-ICE13 XIV 8x8x8 endpoint
</commit_message>
<xml_diff>
--- a/DMC-ICE13/reproduction/seidler_dmc13_recalculation/comparison_workbook.xlsx
+++ b/DMC-ICE13/reproduction/seidler_dmc13_recalculation/comparison_workbook.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re6d9a6786ab844ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch statistics" sheetId="2" r:id="R6913f97e34384634"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relative energies" sheetId="3" r:id="Ra856d74dcc4f452e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch differences" sheetId="4" r:id="R4235f91fa8824f87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absolute parity" sheetId="5" r:id="R1aa348fac95d4862"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Native meshes" sheetId="6" r:id="Rf5db574199884949"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mstore absolute" sheetId="7" r:id="R4f05b190878a4340"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="8" r:id="Rb1915db522b3414e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Reabe28064c9f4899"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch statistics" sheetId="2" r:id="R19074c89ad274ecd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relative energies" sheetId="3" r:id="R28b99a65c7c64fed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch differences" sheetId="4" r:id="Rc54c27faba284aae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absolute parity" sheetId="5" r:id="Rf7071fc64d1445b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Native meshes" sheetId="6" r:id="R4de1317794b244e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mstore absolute" sheetId="7" r:id="R4b23f8a383e84758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="8" r:id="Re9f51ea73f9f442b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -524,7 +524,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb0076e67bc6e4ea6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R228f9dcc45974e94"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1061,7 +1061,7 @@
     <x:mergeCell ref="A24:E24"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84c7269c97fd4b89"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fb42972e9f043d0"/>
 </x:worksheet>
 </file>
 
@@ -3513,25 +3513,25 @@
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
       <x:c r="A81" s="36" t="str">
-        <x:v>author pbc CLI</x:v>
+        <x:v>CP2K-native pbc provider</x:v>
       </x:c>
       <x:c r="B81" s="36" t="str">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C81" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D81" s="42" t="str">
-        <x:v>-40.056162616318</x:v>
+        <x:v>0.090455358961</x:v>
       </x:c>
       <x:c r="E81" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F81" s="42" t="str">
-        <x:v>-40.366162616318</x:v>
+        <x:v>-1.609544641039</x:v>
       </x:c>
       <x:c r="G81" s="42" t="str">
-        <x:v>40.366162616318</x:v>
+        <x:v>1.609544641039</x:v>
       </x:c>
       <x:c r="H81" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3545,19 +3545,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C82" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D82" s="42" t="str">
-        <x:v>-21.728016057439</x:v>
+        <x:v>-40.056162616318</x:v>
       </x:c>
       <x:c r="E82" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F82" s="42" t="str">
-        <x:v>-22.978016057439</x:v>
+        <x:v>-40.366162616318</x:v>
       </x:c>
       <x:c r="G82" s="42" t="str">
-        <x:v>22.978016057439</x:v>
+        <x:v>40.366162616318</x:v>
       </x:c>
       <x:c r="H82" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3571,19 +3571,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C83" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D83" s="42" t="str">
-        <x:v>14.909575775296</x:v>
+        <x:v>-21.728016057439</x:v>
       </x:c>
       <x:c r="E83" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F83" s="42" t="str">
-        <x:v>11.079575775296</x:v>
+        <x:v>-22.978016057439</x:v>
       </x:c>
       <x:c r="G83" s="42" t="str">
-        <x:v>11.079575775296</x:v>
+        <x:v>22.978016057439</x:v>
       </x:c>
       <x:c r="H83" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3597,19 +3597,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C84" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D84" s="42" t="str">
-        <x:v>-57.502753280215</x:v>
+        <x:v>14.909575775296</x:v>
       </x:c>
       <x:c r="E84" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F84" s="42" t="str">
-        <x:v>-59.282753280215</x:v>
+        <x:v>11.079575775296</x:v>
       </x:c>
       <x:c r="G84" s="42" t="str">
-        <x:v>59.282753280215</x:v>
+        <x:v>11.079575775296</x:v>
       </x:c>
       <x:c r="H84" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3623,19 +3623,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C85" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D85" s="42" t="str">
-        <x:v>-300.067320161804</x:v>
+        <x:v>-57.502753280215</x:v>
       </x:c>
       <x:c r="E85" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F85" s="42" t="str">
-        <x:v>-305.057320161804</x:v>
+        <x:v>-59.282753280215</x:v>
       </x:c>
       <x:c r="G85" s="42" t="str">
-        <x:v>305.057320161804</x:v>
+        <x:v>59.282753280215</x:v>
       </x:c>
       <x:c r="H85" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3649,19 +3649,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C86" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D86" s="42" t="str">
-        <x:v>-121.498882525679</x:v>
+        <x:v>-300.067320161804</x:v>
       </x:c>
       <x:c r="E86" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F86" s="42" t="str">
-        <x:v>-125.728882525679</x:v>
+        <x:v>-305.057320161804</x:v>
       </x:c>
       <x:c r="G86" s="42" t="str">
-        <x:v>125.728882525679</x:v>
+        <x:v>305.057320161804</x:v>
       </x:c>
       <x:c r="H86" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3675,19 +3675,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C87" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D87" s="42" t="str">
-        <x:v>-14.812836787859</x:v>
+        <x:v>-121.498882525679</x:v>
       </x:c>
       <x:c r="E87" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F87" s="42" t="str">
-        <x:v>-15.412836787859</x:v>
+        <x:v>-125.728882525679</x:v>
       </x:c>
       <x:c r="G87" s="42" t="str">
-        <x:v>15.412836787859</x:v>
+        <x:v>125.728882525679</x:v>
       </x:c>
       <x:c r="H87" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3701,19 +3701,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C88" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D88" s="42" t="str">
-        <x:v>-165.257377908596</x:v>
+        <x:v>-14.812836787859</x:v>
       </x:c>
       <x:c r="E88" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F88" s="42" t="str">
-        <x:v>-165.417377908596</x:v>
+        <x:v>-15.412836787859</x:v>
       </x:c>
       <x:c r="G88" s="42" t="str">
-        <x:v>165.417377908596</x:v>
+        <x:v>15.412836787859</x:v>
       </x:c>
       <x:c r="H88" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3727,19 +3727,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C89" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D89" s="42" t="str">
-        <x:v>6.868364020212</x:v>
+        <x:v>-165.257377908596</x:v>
       </x:c>
       <x:c r="E89" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F89" s="42" t="str">
-        <x:v>4.748364020212</x:v>
+        <x:v>-165.417377908596</x:v>
       </x:c>
       <x:c r="G89" s="42" t="str">
-        <x:v>4.748364020212</x:v>
+        <x:v>165.417377908596</x:v>
       </x:c>
       <x:c r="H89" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3753,19 +3753,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C90" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D90" s="42" t="str">
-        <x:v>-199.611684777200</x:v>
+        <x:v>6.868364020212</x:v>
       </x:c>
       <x:c r="E90" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F90" s="42" t="str">
-        <x:v>-201.311684777200</x:v>
+        <x:v>4.748364020212</x:v>
       </x:c>
       <x:c r="G90" s="42" t="str">
-        <x:v>201.311684777200</x:v>
+        <x:v>4.748364020212</x:v>
       </x:c>
       <x:c r="H90" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3779,19 +3779,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C91" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D91" s="42" t="str">
-        <x:v>-58.050293332028</x:v>
+        <x:v>-199.611684777200</x:v>
       </x:c>
       <x:c r="E91" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F91" s="42" t="str">
-        <x:v>-59.790293332028</x:v>
+        <x:v>-201.311684777200</x:v>
       </x:c>
       <x:c r="G91" s="42" t="str">
-        <x:v>59.790293332028</x:v>
+        <x:v>201.311684777200</x:v>
       </x:c>
       <x:c r="H91" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3805,19 +3805,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C92" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D92" s="42" t="str">
-        <x:v>-51.559121420866</x:v>
+        <x:v>-58.050293332028</x:v>
       </x:c>
       <x:c r="E92" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F92" s="42" t="str">
-        <x:v>-53.309121420866</x:v>
+        <x:v>-59.790293332028</x:v>
       </x:c>
       <x:c r="G92" s="42" t="str">
-        <x:v>53.309121420866</x:v>
+        <x:v>59.790293332028</x:v>
       </x:c>
       <x:c r="H92" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3828,22 +3828,22 @@
         <x:v>author pbc CLI</x:v>
       </x:c>
       <x:c r="B93" s="36" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C93" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D93" s="42" t="str">
-        <x:v>-9.054674468559</x:v>
+        <x:v>-51.559121420866</x:v>
       </x:c>
       <x:c r="E93" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F93" s="42" t="str">
-        <x:v>-9.364674468559</x:v>
+        <x:v>-53.309121420866</x:v>
       </x:c>
       <x:c r="G93" s="42" t="str">
-        <x:v>9.364674468559</x:v>
+        <x:v>53.309121420866</x:v>
       </x:c>
       <x:c r="H93" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3857,19 +3857,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C94" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D94" s="42" t="str">
-        <x:v>-2.341718734421</x:v>
+        <x:v>-9.054674468559</x:v>
       </x:c>
       <x:c r="E94" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F94" s="42" t="str">
-        <x:v>-3.591718734421</x:v>
+        <x:v>-9.364674468559</x:v>
       </x:c>
       <x:c r="G94" s="42" t="str">
-        <x:v>3.591718734421</x:v>
+        <x:v>9.364674468559</x:v>
       </x:c>
       <x:c r="H94" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3883,19 +3883,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C95" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D95" s="42" t="str">
-        <x:v>2.892295286943</x:v>
+        <x:v>-2.341718734421</x:v>
       </x:c>
       <x:c r="E95" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F95" s="42" t="str">
-        <x:v>-0.937704713057</x:v>
+        <x:v>-3.591718734421</x:v>
       </x:c>
       <x:c r="G95" s="42" t="str">
-        <x:v>0.937704713057</x:v>
+        <x:v>3.591718734421</x:v>
       </x:c>
       <x:c r="H95" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3909,19 +3909,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C96" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D96" s="42" t="str">
-        <x:v>-12.421511801622</x:v>
+        <x:v>2.892295286943</x:v>
       </x:c>
       <x:c r="E96" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F96" s="42" t="str">
-        <x:v>-14.201511801622</x:v>
+        <x:v>-0.937704713057</x:v>
       </x:c>
       <x:c r="G96" s="42" t="str">
-        <x:v>14.201511801622</x:v>
+        <x:v>0.937704713057</x:v>
       </x:c>
       <x:c r="H96" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3935,19 +3935,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C97" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D97" s="42" t="str">
-        <x:v>-153.975297576434</x:v>
+        <x:v>-12.421511801622</x:v>
       </x:c>
       <x:c r="E97" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F97" s="42" t="str">
-        <x:v>-158.965297576434</x:v>
+        <x:v>-14.201511801622</x:v>
       </x:c>
       <x:c r="G97" s="42" t="str">
-        <x:v>158.965297576434</x:v>
+        <x:v>14.201511801622</x:v>
       </x:c>
       <x:c r="H97" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3961,19 +3961,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C98" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D98" s="42" t="str">
-        <x:v>-38.490190110106</x:v>
+        <x:v>-153.975297576434</x:v>
       </x:c>
       <x:c r="E98" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F98" s="42" t="str">
-        <x:v>-42.720190110106</x:v>
+        <x:v>-158.965297576434</x:v>
       </x:c>
       <x:c r="G98" s="42" t="str">
-        <x:v>42.720190110106</x:v>
+        <x:v>158.965297576434</x:v>
       </x:c>
       <x:c r="H98" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3987,19 +3987,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C99" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D99" s="42" t="str">
-        <x:v>-2.462552657305</x:v>
+        <x:v>-38.490190110106</x:v>
       </x:c>
       <x:c r="E99" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F99" s="42" t="str">
-        <x:v>-3.062552657305</x:v>
+        <x:v>-42.720190110106</x:v>
       </x:c>
       <x:c r="G99" s="42" t="str">
-        <x:v>3.062552657305</x:v>
+        <x:v>42.720190110106</x:v>
       </x:c>
       <x:c r="H99" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4013,19 +4013,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C100" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D100" s="42" t="str">
-        <x:v>-62.538655042867</x:v>
+        <x:v>-2.462552657305</x:v>
       </x:c>
       <x:c r="E100" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F100" s="42" t="str">
-        <x:v>-62.698655042867</x:v>
+        <x:v>-3.062552657305</x:v>
       </x:c>
       <x:c r="G100" s="42" t="str">
-        <x:v>62.698655042867</x:v>
+        <x:v>3.062552657305</x:v>
       </x:c>
       <x:c r="H100" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4039,19 +4039,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C101" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D101" s="42" t="str">
-        <x:v>0.923689537732</x:v>
+        <x:v>-62.538655042867</x:v>
       </x:c>
       <x:c r="E101" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F101" s="42" t="str">
-        <x:v>-1.196310462268</x:v>
+        <x:v>-62.698655042867</x:v>
       </x:c>
       <x:c r="G101" s="42" t="str">
-        <x:v>1.196310462268</x:v>
+        <x:v>62.698655042867</x:v>
       </x:c>
       <x:c r="H101" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4065,19 +4065,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C102" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D102" s="42" t="str">
-        <x:v>-83.903026598902</x:v>
+        <x:v>0.923689537732</x:v>
       </x:c>
       <x:c r="E102" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F102" s="42" t="str">
-        <x:v>-85.603026598902</x:v>
+        <x:v>-1.196310462268</x:v>
       </x:c>
       <x:c r="G102" s="42" t="str">
-        <x:v>85.603026598902</x:v>
+        <x:v>1.196310462268</x:v>
       </x:c>
       <x:c r="H102" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4091,19 +4091,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C103" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D103" s="42" t="str">
-        <x:v>-12.548998010281</x:v>
+        <x:v>-83.903026598902</x:v>
       </x:c>
       <x:c r="E103" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F103" s="42" t="str">
-        <x:v>-14.288998010281</x:v>
+        <x:v>-85.603026598902</x:v>
       </x:c>
       <x:c r="G103" s="42" t="str">
-        <x:v>14.288998010281</x:v>
+        <x:v>85.603026598902</x:v>
       </x:c>
       <x:c r="H103" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4117,19 +4117,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C104" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D104" s="42" t="str">
-        <x:v>-10.466416914384</x:v>
+        <x:v>-12.548998010281</x:v>
       </x:c>
       <x:c r="E104" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F104" s="42" t="str">
-        <x:v>-12.216416914384</x:v>
+        <x:v>-14.288998010281</x:v>
       </x:c>
       <x:c r="G104" s="42" t="str">
-        <x:v>12.216416914384</x:v>
+        <x:v>14.288998010281</x:v>
       </x:c>
       <x:c r="H104" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4137,25 +4137,25 @@
     </x:row>
     <x:row r="105" ht="15" hidden="0" customHeight="1">
       <x:c r="A105" s="36" t="str">
-        <x:v>current pbc CLI</x:v>
+        <x:v>author pbc CLI</x:v>
       </x:c>
       <x:c r="B105" s="36" t="str">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C105" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D105" s="42" t="str">
-        <x:v>-85.402832480791</x:v>
+        <x:v>-10.466416914384</x:v>
       </x:c>
       <x:c r="E105" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F105" s="42" t="str">
-        <x:v>-85.712832480791</x:v>
+        <x:v>-12.216416914384</x:v>
       </x:c>
       <x:c r="G105" s="42" t="str">
-        <x:v>85.712832480791</x:v>
+        <x:v>12.216416914384</x:v>
       </x:c>
       <x:c r="H105" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4169,19 +4169,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C106" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D106" s="42" t="str">
-        <x:v>-52.784771448006</x:v>
+        <x:v>-85.402832480791</x:v>
       </x:c>
       <x:c r="E106" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F106" s="42" t="str">
-        <x:v>-54.034771448006</x:v>
+        <x:v>-85.712832480791</x:v>
       </x:c>
       <x:c r="G106" s="42" t="str">
-        <x:v>54.034771448006</x:v>
+        <x:v>85.712832480791</x:v>
       </x:c>
       <x:c r="H106" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4195,19 +4195,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C107" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D107" s="42" t="str">
-        <x:v>38.666296487481</x:v>
+        <x:v>-52.784771448006</x:v>
       </x:c>
       <x:c r="E107" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F107" s="42" t="str">
-        <x:v>34.836296487481</x:v>
+        <x:v>-54.034771448006</x:v>
       </x:c>
       <x:c r="G107" s="42" t="str">
-        <x:v>34.836296487481</x:v>
+        <x:v>54.034771448006</x:v>
       </x:c>
       <x:c r="H107" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4221,19 +4221,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C108" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D108" s="42" t="str">
-        <x:v>-119.951876462899</x:v>
+        <x:v>38.666296487481</x:v>
       </x:c>
       <x:c r="E108" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F108" s="42" t="str">
-        <x:v>-121.731876462899</x:v>
+        <x:v>34.836296487481</x:v>
       </x:c>
       <x:c r="G108" s="42" t="str">
-        <x:v>121.731876462899</x:v>
+        <x:v>34.836296487481</x:v>
       </x:c>
       <x:c r="H108" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4247,19 +4247,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C109" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D109" s="42" t="str">
-        <x:v>-491.873083815613</x:v>
+        <x:v>-119.951876462899</x:v>
       </x:c>
       <x:c r="E109" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F109" s="42" t="str">
-        <x:v>-496.863083815613</x:v>
+        <x:v>-121.731876462899</x:v>
       </x:c>
       <x:c r="G109" s="42" t="str">
-        <x:v>496.863083815613</x:v>
+        <x:v>121.731876462899</x:v>
       </x:c>
       <x:c r="H109" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4273,19 +4273,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C110" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D110" s="42" t="str">
-        <x:v>-227.181421040355</x:v>
+        <x:v>-491.873083815613</x:v>
       </x:c>
       <x:c r="E110" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F110" s="42" t="str">
-        <x:v>-231.411421040355</x:v>
+        <x:v>-496.863083815613</x:v>
       </x:c>
       <x:c r="G110" s="42" t="str">
-        <x:v>231.411421040355</x:v>
+        <x:v>496.863083815613</x:v>
       </x:c>
       <x:c r="H110" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4299,19 +4299,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C111" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D111" s="42" t="str">
-        <x:v>-36.269951925783</x:v>
+        <x:v>-227.181421040355</x:v>
       </x:c>
       <x:c r="E111" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F111" s="42" t="str">
-        <x:v>-36.869951925783</x:v>
+        <x:v>-231.411421040355</x:v>
       </x:c>
       <x:c r="G111" s="42" t="str">
-        <x:v>36.869951925783</x:v>
+        <x:v>231.411421040355</x:v>
       </x:c>
       <x:c r="H111" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4325,19 +4325,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C112" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D112" s="42" t="str">
-        <x:v>-299.258518836626</x:v>
+        <x:v>-36.269951925783</x:v>
       </x:c>
       <x:c r="E112" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F112" s="42" t="str">
-        <x:v>-299.418518836626</x:v>
+        <x:v>-36.869951925783</x:v>
       </x:c>
       <x:c r="G112" s="42" t="str">
-        <x:v>299.418518836626</x:v>
+        <x:v>36.869951925783</x:v>
       </x:c>
       <x:c r="H112" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4351,19 +4351,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C113" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D113" s="42" t="str">
-        <x:v>16.464730608559</x:v>
+        <x:v>-299.258518836626</x:v>
       </x:c>
       <x:c r="E113" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F113" s="42" t="str">
-        <x:v>14.344730608559</x:v>
+        <x:v>-299.418518836626</x:v>
       </x:c>
       <x:c r="G113" s="42" t="str">
-        <x:v>14.344730608559</x:v>
+        <x:v>299.418518836626</x:v>
       </x:c>
       <x:c r="H113" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4377,19 +4377,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C114" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D114" s="42" t="str">
-        <x:v>-351.956576532881</x:v>
+        <x:v>16.464730608559</x:v>
       </x:c>
       <x:c r="E114" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F114" s="42" t="str">
-        <x:v>-353.656576532881</x:v>
+        <x:v>14.344730608559</x:v>
       </x:c>
       <x:c r="G114" s="42" t="str">
-        <x:v>353.656576532881</x:v>
+        <x:v>14.344730608559</x:v>
       </x:c>
       <x:c r="H114" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4403,19 +4403,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C115" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D115" s="42" t="str">
-        <x:v>-121.156628176656</x:v>
+        <x:v>-351.956576532881</x:v>
       </x:c>
       <x:c r="E115" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F115" s="42" t="str">
-        <x:v>-122.896628176656</x:v>
+        <x:v>-353.656576532881</x:v>
       </x:c>
       <x:c r="G115" s="42" t="str">
-        <x:v>122.896628176656</x:v>
+        <x:v>353.656576532881</x:v>
       </x:c>
       <x:c r="H115" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4429,19 +4429,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C116" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D116" s="42" t="str">
-        <x:v>-112.486904450047</x:v>
+        <x:v>-121.156628176656</x:v>
       </x:c>
       <x:c r="E116" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F116" s="42" t="str">
-        <x:v>-114.236904450047</x:v>
+        <x:v>-122.896628176656</x:v>
       </x:c>
       <x:c r="G116" s="42" t="str">
-        <x:v>114.236904450047</x:v>
+        <x:v>122.896628176656</x:v>
       </x:c>
       <x:c r="H116" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4452,22 +4452,22 @@
         <x:v>current pbc CLI</x:v>
       </x:c>
       <x:c r="B117" s="36" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C117" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D117" s="42" t="str">
-        <x:v>-40.052769548562</x:v>
+        <x:v>-112.486904450047</x:v>
       </x:c>
       <x:c r="E117" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F117" s="42" t="str">
-        <x:v>-40.362769548562</x:v>
+        <x:v>-114.236904450047</x:v>
       </x:c>
       <x:c r="G117" s="42" t="str">
-        <x:v>40.362769548562</x:v>
+        <x:v>114.236904450047</x:v>
       </x:c>
       <x:c r="H117" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4481,19 +4481,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C118" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D118" s="42" t="str">
-        <x:v>-21.669458368756</x:v>
+        <x:v>-40.052769548562</x:v>
       </x:c>
       <x:c r="E118" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F118" s="42" t="str">
-        <x:v>-22.919458368756</x:v>
+        <x:v>-40.362769548562</x:v>
       </x:c>
       <x:c r="G118" s="42" t="str">
-        <x:v>22.919458368756</x:v>
+        <x:v>40.362769548562</x:v>
       </x:c>
       <x:c r="H118" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4507,19 +4507,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C119" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D119" s="42" t="str">
-        <x:v>14.926647908813</x:v>
+        <x:v>-21.669458368756</x:v>
       </x:c>
       <x:c r="E119" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F119" s="42" t="str">
-        <x:v>11.096647908813</x:v>
+        <x:v>-22.919458368756</x:v>
       </x:c>
       <x:c r="G119" s="42" t="str">
-        <x:v>11.096647908813</x:v>
+        <x:v>22.919458368756</x:v>
       </x:c>
       <x:c r="H119" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4533,19 +4533,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C120" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D120" s="42" t="str">
-        <x:v>-57.367276074495</x:v>
+        <x:v>14.926647908813</x:v>
       </x:c>
       <x:c r="E120" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F120" s="42" t="str">
-        <x:v>-59.147276074495</x:v>
+        <x:v>11.096647908813</x:v>
       </x:c>
       <x:c r="G120" s="42" t="str">
-        <x:v>59.147276074495</x:v>
+        <x:v>11.096647908813</x:v>
       </x:c>
       <x:c r="H120" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4559,19 +4559,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C121" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D121" s="42" t="str">
-        <x:v>-299.975204903283</x:v>
+        <x:v>-57.367276074495</x:v>
       </x:c>
       <x:c r="E121" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F121" s="42" t="str">
-        <x:v>-304.965204903283</x:v>
+        <x:v>-59.147276074495</x:v>
       </x:c>
       <x:c r="G121" s="42" t="str">
-        <x:v>304.965204903283</x:v>
+        <x:v>59.147276074495</x:v>
       </x:c>
       <x:c r="H121" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4585,19 +4585,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C122" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D122" s="42" t="str">
-        <x:v>-121.493623038083</x:v>
+        <x:v>-299.975204903283</x:v>
       </x:c>
       <x:c r="E122" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F122" s="42" t="str">
-        <x:v>-125.723623038083</x:v>
+        <x:v>-304.965204903283</x:v>
       </x:c>
       <x:c r="G122" s="42" t="str">
-        <x:v>125.723623038083</x:v>
+        <x:v>304.965204903283</x:v>
       </x:c>
       <x:c r="H122" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4611,19 +4611,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C123" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D123" s="42" t="str">
-        <x:v>-14.811033266160</x:v>
+        <x:v>-121.493623038083</x:v>
       </x:c>
       <x:c r="E123" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F123" s="42" t="str">
-        <x:v>-15.411033266160</x:v>
+        <x:v>-125.723623038083</x:v>
       </x:c>
       <x:c r="G123" s="42" t="str">
-        <x:v>15.411033266160</x:v>
+        <x:v>125.723623038083</x:v>
       </x:c>
       <x:c r="H123" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4637,19 +4637,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C124" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D124" s="42" t="str">
-        <x:v>-165.236809268426</x:v>
+        <x:v>-14.811033266160</x:v>
       </x:c>
       <x:c r="E124" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F124" s="42" t="str">
-        <x:v>-165.396809268426</x:v>
+        <x:v>-15.411033266160</x:v>
       </x:c>
       <x:c r="G124" s="42" t="str">
-        <x:v>165.396809268426</x:v>
+        <x:v>15.411033266160</x:v>
       </x:c>
       <x:c r="H124" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4663,19 +4663,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C125" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D125" s="42" t="str">
-        <x:v>6.872357662713</x:v>
+        <x:v>-165.236809268426</x:v>
       </x:c>
       <x:c r="E125" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F125" s="42" t="str">
-        <x:v>4.752357662713</x:v>
+        <x:v>-165.396809268426</x:v>
       </x:c>
       <x:c r="G125" s="42" t="str">
-        <x:v>4.752357662713</x:v>
+        <x:v>165.396809268426</x:v>
       </x:c>
       <x:c r="H125" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4689,19 +4689,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C126" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D126" s="42" t="str">
-        <x:v>-199.607041791688</x:v>
+        <x:v>6.872357662713</x:v>
       </x:c>
       <x:c r="E126" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F126" s="42" t="str">
-        <x:v>-201.307041791688</x:v>
+        <x:v>4.752357662713</x:v>
       </x:c>
       <x:c r="G126" s="42" t="str">
-        <x:v>201.307041791688</x:v>
+        <x:v>4.752357662713</x:v>
       </x:c>
       <x:c r="H126" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4715,19 +4715,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C127" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D127" s="42" t="str">
-        <x:v>-58.045564075785</x:v>
+        <x:v>-199.607041791688</x:v>
       </x:c>
       <x:c r="E127" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F127" s="42" t="str">
-        <x:v>-59.785564075785</x:v>
+        <x:v>-201.307041791688</x:v>
       </x:c>
       <x:c r="G127" s="42" t="str">
-        <x:v>59.785564075785</x:v>
+        <x:v>201.307041791688</x:v>
       </x:c>
       <x:c r="H127" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4741,19 +4741,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C128" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D128" s="42" t="str">
-        <x:v>-51.558720983607</x:v>
+        <x:v>-58.045564075785</x:v>
       </x:c>
       <x:c r="E128" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F128" s="42" t="str">
-        <x:v>-53.308720983607</x:v>
+        <x:v>-59.785564075785</x:v>
       </x:c>
       <x:c r="G128" s="42" t="str">
-        <x:v>53.308720983607</x:v>
+        <x:v>59.785564075785</x:v>
       </x:c>
       <x:c r="H128" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4764,22 +4764,22 @@
         <x:v>current pbc CLI</x:v>
       </x:c>
       <x:c r="B129" s="36" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C129" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D129" s="42" t="str">
-        <x:v>-9.052128552229</x:v>
+        <x:v>-51.558720983607</x:v>
       </x:c>
       <x:c r="E129" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F129" s="42" t="str">
-        <x:v>-9.362128552229</x:v>
+        <x:v>-53.308720983607</x:v>
       </x:c>
       <x:c r="G129" s="42" t="str">
-        <x:v>9.362128552229</x:v>
+        <x:v>53.308720983607</x:v>
       </x:c>
       <x:c r="H129" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4793,19 +4793,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C130" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D130" s="42" t="str">
-        <x:v>-2.299617048110</x:v>
+        <x:v>-9.052128552229</x:v>
       </x:c>
       <x:c r="E130" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F130" s="42" t="str">
-        <x:v>-3.549617048110</x:v>
+        <x:v>-9.362128552229</x:v>
       </x:c>
       <x:c r="G130" s="42" t="str">
-        <x:v>3.549617048110</x:v>
+        <x:v>9.362128552229</x:v>
       </x:c>
       <x:c r="H130" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4819,19 +4819,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C131" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D131" s="42" t="str">
-        <x:v>2.904340310370</x:v>
+        <x:v>-2.299617048110</x:v>
       </x:c>
       <x:c r="E131" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F131" s="42" t="str">
-        <x:v>-0.925659689630</x:v>
+        <x:v>-3.549617048110</x:v>
       </x:c>
       <x:c r="G131" s="42" t="str">
-        <x:v>0.925659689630</x:v>
+        <x:v>3.549617048110</x:v>
       </x:c>
       <x:c r="H131" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4845,19 +4845,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C132" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D132" s="42" t="str">
-        <x:v>-12.321031303355</x:v>
+        <x:v>2.904340310370</x:v>
       </x:c>
       <x:c r="E132" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F132" s="42" t="str">
-        <x:v>-14.101031303355</x:v>
+        <x:v>-0.925659689630</x:v>
       </x:c>
       <x:c r="G132" s="42" t="str">
-        <x:v>14.101031303355</x:v>
+        <x:v>0.925659689630</x:v>
       </x:c>
       <x:c r="H132" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4871,19 +4871,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C133" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D133" s="42" t="str">
-        <x:v>-153.898129900577</x:v>
+        <x:v>-12.321031303355</x:v>
       </x:c>
       <x:c r="E133" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F133" s="42" t="str">
-        <x:v>-158.888129900577</x:v>
+        <x:v>-14.101031303355</x:v>
       </x:c>
       <x:c r="G133" s="42" t="str">
-        <x:v>158.888129900577</x:v>
+        <x:v>14.101031303355</x:v>
       </x:c>
       <x:c r="H133" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4897,19 +4897,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C134" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D134" s="42" t="str">
-        <x:v>-38.486266197120</x:v>
+        <x:v>-153.898129900577</x:v>
       </x:c>
       <x:c r="E134" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F134" s="42" t="str">
-        <x:v>-42.716266197120</x:v>
+        <x:v>-158.888129900577</x:v>
       </x:c>
       <x:c r="G134" s="42" t="str">
-        <x:v>42.716266197120</x:v>
+        <x:v>158.888129900577</x:v>
       </x:c>
       <x:c r="H134" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4923,19 +4923,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C135" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D135" s="42" t="str">
-        <x:v>-2.461004071112</x:v>
+        <x:v>-38.486266197120</x:v>
       </x:c>
       <x:c r="E135" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F135" s="42" t="str">
-        <x:v>-3.061004071112</x:v>
+        <x:v>-42.716266197120</x:v>
       </x:c>
       <x:c r="G135" s="42" t="str">
-        <x:v>3.061004071112</x:v>
+        <x:v>42.716266197120</x:v>
       </x:c>
       <x:c r="H135" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4949,19 +4949,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C136" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D136" s="42" t="str">
-        <x:v>-62.523175264048</x:v>
+        <x:v>-2.461004071112</x:v>
       </x:c>
       <x:c r="E136" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F136" s="42" t="str">
-        <x:v>-62.683175264048</x:v>
+        <x:v>-3.061004071112</x:v>
       </x:c>
       <x:c r="G136" s="42" t="str">
-        <x:v>62.683175264048</x:v>
+        <x:v>3.061004071112</x:v>
       </x:c>
       <x:c r="H136" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4975,19 +4975,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C137" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D137" s="42" t="str">
-        <x:v>0.926723486584</x:v>
+        <x:v>-62.523175264048</x:v>
       </x:c>
       <x:c r="E137" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F137" s="42" t="str">
-        <x:v>-1.193276513416</x:v>
+        <x:v>-62.683175264048</x:v>
       </x:c>
       <x:c r="G137" s="42" t="str">
-        <x:v>1.193276513416</x:v>
+        <x:v>62.683175264048</x:v>
       </x:c>
       <x:c r="H137" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5001,19 +5001,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C138" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D138" s="42" t="str">
-        <x:v>-83.899718986935</x:v>
+        <x:v>0.926723486584</x:v>
       </x:c>
       <x:c r="E138" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F138" s="42" t="str">
-        <x:v>-85.599718986935</x:v>
+        <x:v>-1.193276513416</x:v>
       </x:c>
       <x:c r="G138" s="42" t="str">
-        <x:v>85.599718986935</x:v>
+        <x:v>1.193276513416</x:v>
       </x:c>
       <x:c r="H138" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5027,19 +5027,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C139" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D139" s="42" t="str">
-        <x:v>-12.545503073689</x:v>
+        <x:v>-83.899718986935</x:v>
       </x:c>
       <x:c r="E139" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F139" s="42" t="str">
-        <x:v>-14.285503073689</x:v>
+        <x:v>-85.599718986935</x:v>
       </x:c>
       <x:c r="G139" s="42" t="str">
-        <x:v>14.285503073689</x:v>
+        <x:v>85.599718986935</x:v>
       </x:c>
       <x:c r="H139" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5053,19 +5053,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C140" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D140" s="42" t="str">
-        <x:v>-10.466391957817</x:v>
+        <x:v>-12.545503073689</x:v>
       </x:c>
       <x:c r="E140" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F140" s="42" t="str">
-        <x:v>-12.216391957817</x:v>
+        <x:v>-14.285503073689</x:v>
       </x:c>
       <x:c r="G140" s="42" t="str">
-        <x:v>12.216391957817</x:v>
+        <x:v>14.285503073689</x:v>
       </x:c>
       <x:c r="H140" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5076,22 +5076,22 @@
         <x:v>current pbc CLI</x:v>
       </x:c>
       <x:c r="B141" s="36" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C141" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D141" s="42" t="str">
-        <x:v>-2.513150603252</x:v>
+        <x:v>-10.466391957817</x:v>
       </x:c>
       <x:c r="E141" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F141" s="42" t="str">
-        <x:v>-2.823150603252</x:v>
+        <x:v>-12.216391957817</x:v>
       </x:c>
       <x:c r="G141" s="42" t="str">
-        <x:v>2.823150603252</x:v>
+        <x:v>12.216391957817</x:v>
       </x:c>
       <x:c r="H141" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5105,19 +5105,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C142" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D142" s="42" t="str">
-        <x:v>1.264029937698</x:v>
+        <x:v>-2.513150603252</x:v>
       </x:c>
       <x:c r="E142" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F142" s="42" t="str">
-        <x:v>0.014029937698</x:v>
+        <x:v>-2.823150603252</x:v>
       </x:c>
       <x:c r="G142" s="42" t="str">
-        <x:v>0.014029937698</x:v>
+        <x:v>2.823150603252</x:v>
       </x:c>
       <x:c r="H142" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5131,19 +5131,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C143" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D143" s="42" t="str">
-        <x:v>1.405712159485</x:v>
+        <x:v>1.264029937698</x:v>
       </x:c>
       <x:c r="E143" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F143" s="42" t="str">
-        <x:v>-2.424287840515</x:v>
+        <x:v>0.014029937698</x:v>
       </x:c>
       <x:c r="G143" s="42" t="str">
-        <x:v>2.424287840515</x:v>
+        <x:v>0.014029937698</x:v>
       </x:c>
       <x:c r="H143" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5157,19 +5157,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C144" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D144" s="42" t="str">
-        <x:v>-1.048061577331</x:v>
+        <x:v>1.405712159485</x:v>
       </x:c>
       <x:c r="E144" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F144" s="42" t="str">
-        <x:v>-2.828061577331</x:v>
+        <x:v>-2.424287840515</x:v>
       </x:c>
       <x:c r="G144" s="42" t="str">
-        <x:v>2.828061577331</x:v>
+        <x:v>2.424287840515</x:v>
       </x:c>
       <x:c r="H144" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5183,19 +5183,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C145" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D145" s="42" t="str">
-        <x:v>-63.955235096392</x:v>
+        <x:v>-1.048061577331</x:v>
       </x:c>
       <x:c r="E145" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F145" s="42" t="str">
-        <x:v>-68.945235096392</x:v>
+        <x:v>-2.828061577331</x:v>
       </x:c>
       <x:c r="G145" s="42" t="str">
-        <x:v>68.945235096392</x:v>
+        <x:v>2.828061577331</x:v>
       </x:c>
       <x:c r="H145" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5209,19 +5209,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C146" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D146" s="42" t="str">
-        <x:v>-6.163484047291</x:v>
+        <x:v>-63.955235096392</x:v>
       </x:c>
       <x:c r="E146" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F146" s="42" t="str">
-        <x:v>-10.393484047291</x:v>
+        <x:v>-68.945235096392</x:v>
       </x:c>
       <x:c r="G146" s="42" t="str">
-        <x:v>10.393484047291</x:v>
+        <x:v>68.945235096392</x:v>
       </x:c>
       <x:c r="H146" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5235,19 +5235,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C147" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D147" s="42" t="str">
-        <x:v>-0.372876272237</x:v>
+        <x:v>-6.163484047291</x:v>
       </x:c>
       <x:c r="E147" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F147" s="42" t="str">
-        <x:v>-0.972876272237</x:v>
+        <x:v>-10.393484047291</x:v>
       </x:c>
       <x:c r="G147" s="42" t="str">
-        <x:v>0.972876272237</x:v>
+        <x:v>10.393484047291</x:v>
       </x:c>
       <x:c r="H147" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5261,19 +5261,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C148" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D148" s="42" t="str">
-        <x:v>-14.875013200229</x:v>
+        <x:v>-0.372876272237</x:v>
       </x:c>
       <x:c r="E148" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F148" s="42" t="str">
-        <x:v>-15.035013200229</x:v>
+        <x:v>-0.972876272237</x:v>
       </x:c>
       <x:c r="G148" s="42" t="str">
-        <x:v>15.035013200229</x:v>
+        <x:v>0.972876272237</x:v>
       </x:c>
       <x:c r="H148" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5287,19 +5287,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C149" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D149" s="42" t="str">
-        <x:v>0.123061371006</x:v>
+        <x:v>-14.875013200229</x:v>
       </x:c>
       <x:c r="E149" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F149" s="42" t="str">
-        <x:v>-1.996938628994</x:v>
+        <x:v>-15.035013200229</x:v>
       </x:c>
       <x:c r="G149" s="42" t="str">
-        <x:v>1.996938628994</x:v>
+        <x:v>15.035013200229</x:v>
       </x:c>
       <x:c r="H149" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5313,19 +5313,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C150" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D150" s="42" t="str">
-        <x:v>-23.938106879109</x:v>
+        <x:v>0.123061371006</x:v>
       </x:c>
       <x:c r="E150" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F150" s="42" t="str">
-        <x:v>-25.638106879109</x:v>
+        <x:v>-1.996938628994</x:v>
       </x:c>
       <x:c r="G150" s="42" t="str">
-        <x:v>25.638106879109</x:v>
+        <x:v>1.996938628994</x:v>
       </x:c>
       <x:c r="H150" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5339,19 +5339,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C151" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D151" s="42" t="str">
-        <x:v>-1.097393985422</x:v>
+        <x:v>-23.938106879109</x:v>
       </x:c>
       <x:c r="E151" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F151" s="42" t="str">
-        <x:v>-2.837393985422</x:v>
+        <x:v>-25.638106879109</x:v>
       </x:c>
       <x:c r="G151" s="42" t="str">
-        <x:v>2.837393985422</x:v>
+        <x:v>25.638106879109</x:v>
       </x:c>
       <x:c r="H151" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5365,19 +5365,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C152" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D152" s="42" t="str">
-        <x:v>-0.727230275074</x:v>
+        <x:v>-1.097393985422</x:v>
       </x:c>
       <x:c r="E152" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F152" s="42" t="str">
-        <x:v>-2.477230275074</x:v>
+        <x:v>-2.837393985422</x:v>
       </x:c>
       <x:c r="G152" s="42" t="str">
-        <x:v>2.477230275074</x:v>
+        <x:v>2.837393985422</x:v>
       </x:c>
       <x:c r="H152" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5385,25 +5385,25 @@
     </x:row>
     <x:row r="153" ht="15" hidden="0" customHeight="1">
       <x:c r="A153" s="36" t="str">
-        <x:v>historical mstore-inorganic CLI</x:v>
+        <x:v>current pbc CLI</x:v>
       </x:c>
       <x:c r="B153" s="36" t="str">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C153" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D153" s="42" t="str">
-        <x:v>11.549596417487</x:v>
+        <x:v>-0.727230275074</x:v>
       </x:c>
       <x:c r="E153" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F153" s="42" t="str">
-        <x:v>11.239596417487</x:v>
+        <x:v>-2.477230275074</x:v>
       </x:c>
       <x:c r="G153" s="42" t="str">
-        <x:v>11.239596417487</x:v>
+        <x:v>2.477230275074</x:v>
       </x:c>
       <x:c r="H153" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5417,19 +5417,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C154" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D154" s="42" t="str">
-        <x:v>-29.811523391510</x:v>
+        <x:v>11.549596417487</x:v>
       </x:c>
       <x:c r="E154" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F154" s="42" t="str">
-        <x:v>-31.061523391510</x:v>
+        <x:v>11.239596417487</x:v>
       </x:c>
       <x:c r="G154" s="42" t="str">
-        <x:v>31.061523391510</x:v>
+        <x:v>11.239596417487</x:v>
       </x:c>
       <x:c r="H154" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5443,19 +5443,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C155" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D155" s="42" t="str">
-        <x:v>0.256599145141</x:v>
+        <x:v>-29.811523391510</x:v>
       </x:c>
       <x:c r="E155" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F155" s="42" t="str">
-        <x:v>-3.573400854859</x:v>
+        <x:v>-31.061523391510</x:v>
       </x:c>
       <x:c r="G155" s="42" t="str">
-        <x:v>3.573400854859</x:v>
+        <x:v>31.061523391510</x:v>
       </x:c>
       <x:c r="H155" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5469,19 +5469,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C156" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D156" s="42" t="str">
-        <x:v>-28.460677817350</x:v>
+        <x:v>0.256599145141</x:v>
       </x:c>
       <x:c r="E156" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F156" s="42" t="str">
-        <x:v>-30.240677817350</x:v>
+        <x:v>-3.573400854859</x:v>
       </x:c>
       <x:c r="G156" s="42" t="str">
-        <x:v>30.240677817350</x:v>
+        <x:v>3.573400854859</x:v>
       </x:c>
       <x:c r="H156" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5495,19 +5495,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C157" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D157" s="42" t="str">
-        <x:v>-151.947965741842</x:v>
+        <x:v>-28.460677817350</x:v>
       </x:c>
       <x:c r="E157" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F157" s="42" t="str">
-        <x:v>-156.937965741842</x:v>
+        <x:v>-30.240677817350</x:v>
       </x:c>
       <x:c r="G157" s="42" t="str">
-        <x:v>156.937965741842</x:v>
+        <x:v>30.240677817350</x:v>
       </x:c>
       <x:c r="H157" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5521,19 +5521,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C158" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D158" s="42" t="str">
-        <x:v>-77.417542603032</x:v>
+        <x:v>-151.947965741842</x:v>
       </x:c>
       <x:c r="E158" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F158" s="42" t="str">
-        <x:v>-81.647542603032</x:v>
+        <x:v>-156.937965741842</x:v>
       </x:c>
       <x:c r="G158" s="42" t="str">
-        <x:v>81.647542603032</x:v>
+        <x:v>156.937965741842</x:v>
       </x:c>
       <x:c r="H158" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5547,19 +5547,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C159" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D159" s="42" t="str">
-        <x:v>-24.470250890265</x:v>
+        <x:v>-77.417542603032</x:v>
       </x:c>
       <x:c r="E159" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F159" s="42" t="str">
-        <x:v>-25.070250890265</x:v>
+        <x:v>-81.647542603032</x:v>
       </x:c>
       <x:c r="G159" s="42" t="str">
-        <x:v>25.070250890265</x:v>
+        <x:v>81.647542603032</x:v>
       </x:c>
       <x:c r="H159" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5573,19 +5573,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C160" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D160" s="42" t="str">
-        <x:v>-84.549975905731</x:v>
+        <x:v>-24.470250890265</x:v>
       </x:c>
       <x:c r="E160" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F160" s="42" t="str">
-        <x:v>-84.709975905731</x:v>
+        <x:v>-25.070250890265</x:v>
       </x:c>
       <x:c r="G160" s="42" t="str">
-        <x:v>84.709975905731</x:v>
+        <x:v>25.070250890265</x:v>
       </x:c>
       <x:c r="H160" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5599,19 +5599,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C161" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D161" s="42" t="str">
-        <x:v>0.922244833924</x:v>
+        <x:v>-84.549975905731</x:v>
       </x:c>
       <x:c r="E161" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F161" s="42" t="str">
-        <x:v>-1.197755166076</x:v>
+        <x:v>-84.709975905731</x:v>
       </x:c>
       <x:c r="G161" s="42" t="str">
-        <x:v>1.197755166076</x:v>
+        <x:v>84.709975905731</x:v>
       </x:c>
       <x:c r="H161" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5625,19 +5625,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C162" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D162" s="42" t="str">
-        <x:v>-99.557194036284</x:v>
+        <x:v>0.922244833924</x:v>
       </x:c>
       <x:c r="E162" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F162" s="42" t="str">
-        <x:v>-101.257194036284</x:v>
+        <x:v>-1.197755166076</x:v>
       </x:c>
       <x:c r="G162" s="42" t="str">
-        <x:v>101.257194036284</x:v>
+        <x:v>1.197755166076</x:v>
       </x:c>
       <x:c r="H162" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5651,19 +5651,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C163" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D163" s="42" t="str">
-        <x:v>-28.664951204286</x:v>
+        <x:v>-99.557194036284</x:v>
       </x:c>
       <x:c r="E163" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F163" s="42" t="str">
-        <x:v>-30.404951204286</x:v>
+        <x:v>-101.257194036284</x:v>
       </x:c>
       <x:c r="G163" s="42" t="str">
-        <x:v>30.404951204286</x:v>
+        <x:v>101.257194036284</x:v>
       </x:c>
       <x:c r="H163" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5677,19 +5677,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C164" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D164" s="42" t="str">
-        <x:v>-25.438330429983</x:v>
+        <x:v>-28.664951204286</x:v>
       </x:c>
       <x:c r="E164" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F164" s="42" t="str">
-        <x:v>-27.188330429983</x:v>
+        <x:v>-30.404951204286</x:v>
       </x:c>
       <x:c r="G164" s="42" t="str">
-        <x:v>27.188330429983</x:v>
+        <x:v>30.404951204286</x:v>
       </x:c>
       <x:c r="H164" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5700,22 +5700,22 @@
         <x:v>historical mstore-inorganic CLI</x:v>
       </x:c>
       <x:c r="B165" s="36" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C165" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D165" s="42" t="str">
-        <x:v>-0.279988209907</x:v>
+        <x:v>-25.438330429983</x:v>
       </x:c>
       <x:c r="E165" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F165" s="42" t="str">
-        <x:v>-0.589988209907</x:v>
+        <x:v>-27.188330429983</x:v>
       </x:c>
       <x:c r="G165" s="42" t="str">
-        <x:v>0.589988209907</x:v>
+        <x:v>27.188330429983</x:v>
       </x:c>
       <x:c r="H165" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5729,19 +5729,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C166" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D166" s="42" t="str">
-        <x:v>-1.720202220170</x:v>
+        <x:v>-0.279988209907</x:v>
       </x:c>
       <x:c r="E166" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F166" s="42" t="str">
-        <x:v>-2.970202220170</x:v>
+        <x:v>-0.589988209907</x:v>
       </x:c>
       <x:c r="G166" s="42" t="str">
-        <x:v>2.970202220170</x:v>
+        <x:v>0.589988209907</x:v>
       </x:c>
       <x:c r="H166" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5755,19 +5755,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C167" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D167" s="42" t="str">
-        <x:v>1.653583137544</x:v>
+        <x:v>-1.720202220170</x:v>
       </x:c>
       <x:c r="E167" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F167" s="42" t="str">
-        <x:v>-2.176416862456</x:v>
+        <x:v>-2.970202220170</x:v>
       </x:c>
       <x:c r="G167" s="42" t="str">
-        <x:v>2.176416862456</x:v>
+        <x:v>2.970202220170</x:v>
       </x:c>
       <x:c r="H167" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5781,19 +5781,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C168" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D168" s="42" t="str">
-        <x:v>-5.912105883998</x:v>
+        <x:v>1.653583137544</x:v>
       </x:c>
       <x:c r="E168" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F168" s="42" t="str">
-        <x:v>-7.692105883998</x:v>
+        <x:v>-2.176416862456</x:v>
       </x:c>
       <x:c r="G168" s="42" t="str">
-        <x:v>7.692105883998</x:v>
+        <x:v>2.176416862456</x:v>
       </x:c>
       <x:c r="H168" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5807,19 +5807,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C169" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D169" s="42" t="str">
-        <x:v>-77.446667006181</x:v>
+        <x:v>-5.912105883998</x:v>
       </x:c>
       <x:c r="E169" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F169" s="42" t="str">
-        <x:v>-82.436667006181</x:v>
+        <x:v>-7.692105883998</x:v>
       </x:c>
       <x:c r="G169" s="42" t="str">
-        <x:v>82.436667006181</x:v>
+        <x:v>7.692105883998</x:v>
       </x:c>
       <x:c r="H169" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5833,19 +5833,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C170" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D170" s="42" t="str">
-        <x:v>-19.706722185486</x:v>
+        <x:v>-77.446667006181</x:v>
       </x:c>
       <x:c r="E170" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F170" s="42" t="str">
-        <x:v>-23.936722185486</x:v>
+        <x:v>-82.436667006181</x:v>
       </x:c>
       <x:c r="G170" s="42" t="str">
-        <x:v>23.936722185486</x:v>
+        <x:v>82.436667006181</x:v>
       </x:c>
       <x:c r="H170" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5859,19 +5859,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C171" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D171" s="42" t="str">
-        <x:v>-2.774771626398</x:v>
+        <x:v>-19.706722185486</x:v>
       </x:c>
       <x:c r="E171" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F171" s="42" t="str">
-        <x:v>-3.374771626398</x:v>
+        <x:v>-23.936722185486</x:v>
       </x:c>
       <x:c r="G171" s="42" t="str">
-        <x:v>3.374771626398</x:v>
+        <x:v>23.936722185486</x:v>
       </x:c>
       <x:c r="H171" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5885,19 +5885,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C172" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D172" s="42" t="str">
-        <x:v>-31.168750655955</x:v>
+        <x:v>-2.774771626398</x:v>
       </x:c>
       <x:c r="E172" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F172" s="42" t="str">
-        <x:v>-31.328750655955</x:v>
+        <x:v>-3.374771626398</x:v>
       </x:c>
       <x:c r="G172" s="42" t="str">
-        <x:v>31.328750655955</x:v>
+        <x:v>3.374771626398</x:v>
       </x:c>
       <x:c r="H172" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5911,19 +5911,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C173" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D173" s="42" t="str">
-        <x:v>0.442953962487</x:v>
+        <x:v>-31.168750655955</x:v>
       </x:c>
       <x:c r="E173" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F173" s="42" t="str">
-        <x:v>-1.677046037513</x:v>
+        <x:v>-31.328750655955</x:v>
       </x:c>
       <x:c r="G173" s="42" t="str">
-        <x:v>1.677046037513</x:v>
+        <x:v>31.328750655955</x:v>
       </x:c>
       <x:c r="H173" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5937,19 +5937,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C174" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D174" s="42" t="str">
-        <x:v>-41.779791859131</x:v>
+        <x:v>0.442953962487</x:v>
       </x:c>
       <x:c r="E174" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F174" s="42" t="str">
-        <x:v>-43.479791859131</x:v>
+        <x:v>-1.677046037513</x:v>
       </x:c>
       <x:c r="G174" s="42" t="str">
-        <x:v>43.479791859131</x:v>
+        <x:v>1.677046037513</x:v>
       </x:c>
       <x:c r="H174" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5963,19 +5963,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C175" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D175" s="42" t="str">
-        <x:v>-5.934441749535</x:v>
+        <x:v>-41.779791859131</x:v>
       </x:c>
       <x:c r="E175" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F175" s="42" t="str">
-        <x:v>-7.674441749535</x:v>
+        <x:v>-43.479791859131</x:v>
       </x:c>
       <x:c r="G175" s="42" t="str">
-        <x:v>7.674441749535</x:v>
+        <x:v>43.479791859131</x:v>
       </x:c>
       <x:c r="H175" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5989,21 +5989,47 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C176" s="36" t="str">
+        <x:v>XV</x:v>
+      </x:c>
+      <x:c r="D176" s="42" t="str">
+        <x:v>-5.934441749535</x:v>
+      </x:c>
+      <x:c r="E176" s="42" t="str">
+        <x:v>1.740000</x:v>
+      </x:c>
+      <x:c r="F176" s="42" t="str">
+        <x:v>-7.674441749535</x:v>
+      </x:c>
+      <x:c r="G176" s="42" t="str">
+        <x:v>7.674441749535</x:v>
+      </x:c>
+      <x:c r="H176" s="36" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="15" hidden="0" customHeight="1">
+      <x:c r="A177" s="36" t="str">
+        <x:v>historical mstore-inorganic CLI</x:v>
+      </x:c>
+      <x:c r="B177" s="36" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C177" s="36" t="str">
         <x:v>XVII</x:v>
       </x:c>
-      <x:c r="D176" s="42" t="str">
+      <x:c r="D177" s="42" t="str">
         <x:v>-4.880577524129</x:v>
       </x:c>
-      <x:c r="E176" s="42" t="str">
+      <x:c r="E177" s="42" t="str">
         <x:v>1.750000</x:v>
       </x:c>
-      <x:c r="F176" s="42" t="str">
+      <x:c r="F177" s="42" t="str">
         <x:v>-6.630577524129</x:v>
       </x:c>
-      <x:c r="G176" s="42" t="str">
+      <x:c r="G177" s="42" t="str">
         <x:v>6.630577524129</x:v>
       </x:c>
-      <x:c r="H176" s="36" t="str">
+      <x:c r="H177" s="36" t="str">
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
@@ -10892,6 +10918,32 @@
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
+    <x:row r="81" ht="15" hidden="0" customHeight="1">
+      <x:c r="A81" s="36" t="str">
+        <x:v>CP2K-native pbc provider</x:v>
+      </x:c>
+      <x:c r="B81" s="36" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C81" s="36" t="str">
+        <x:v>XIV</x:v>
+      </x:c>
+      <x:c r="D81" s="42" t="str">
+        <x:v>0.090455358961</x:v>
+      </x:c>
+      <x:c r="E81" s="42" t="str">
+        <x:v>1.700000</x:v>
+      </x:c>
+      <x:c r="F81" s="42" t="str">
+        <x:v>-1.609544641039</x:v>
+      </x:c>
+      <x:c r="G81" s="42" t="str">
+        <x:v>1.609544641039</x:v>
+      </x:c>
+      <x:c r="H81" s="36" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Archive qualified XI 8x8x8 and refresh Part I
</commit_message>
<xml_diff>
--- a/DMC-ICE13/reproduction/seidler_dmc13_recalculation/comparison_workbook.xlsx
+++ b/DMC-ICE13/reproduction/seidler_dmc13_recalculation/comparison_workbook.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R143bfb9c0f194c1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch statistics" sheetId="2" r:id="Red175082568a434f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relative energies" sheetId="3" r:id="R42a0f59b0a554140"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch differences" sheetId="4" r:id="Rfef6cab5e87149a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absolute parity" sheetId="5" r:id="Rda6b4d1b66c04a20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Native meshes" sheetId="6" r:id="Rdfee209259314721"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mstore absolute" sheetId="7" r:id="R2a51f1bdebd24f70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="8" r:id="R76beba646cb74d32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb666662d441b48b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch statistics" sheetId="2" r:id="R9c366c3a849347a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relative energies" sheetId="3" r:id="R990069d02d2d4e2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch differences" sheetId="4" r:id="Re562defc59124850"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Absolute parity" sheetId="5" r:id="Rbeee38ce48434b18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Native meshes" sheetId="6" r:id="Ree91b4f30a4e42ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mstore absolute" sheetId="7" r:id="Rffd01ef99f3f4a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="References" sheetId="8" r:id="Rbae01682e9314cdc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -524,7 +524,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0d786a217f1641c7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R13a613f211174a69"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1079,7 +1079,7 @@
     <x:mergeCell ref="A24:E24"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1baf0f69a85426e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89d0416fc1d14cdb"/>
 </x:worksheet>
 </file>
 
@@ -3586,19 +3586,19 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C82" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D82" s="42" t="str">
-        <x:v>0.090455358961</x:v>
+        <x:v>0.508805411655</x:v>
       </x:c>
       <x:c r="E82" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F82" s="42" t="str">
-        <x:v>-1.609544641039</x:v>
+        <x:v>0.348805411655</x:v>
       </x:c>
       <x:c r="G82" s="42" t="str">
-        <x:v>1.609544641039</x:v>
+        <x:v>0.348805411655</x:v>
       </x:c>
       <x:c r="H82" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3606,25 +3606,25 @@
     </x:row>
     <x:row r="83" ht="15" hidden="0" customHeight="1">
       <x:c r="A83" s="36" t="str">
-        <x:v>author pbc CLI</x:v>
+        <x:v>CP2K-native pbc provider</x:v>
       </x:c>
       <x:c r="B83" s="36" t="str">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C83" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D83" s="42" t="str">
-        <x:v>-40.056162616318</x:v>
+        <x:v>0.090455358961</x:v>
       </x:c>
       <x:c r="E83" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F83" s="42" t="str">
-        <x:v>-40.366162616318</x:v>
+        <x:v>-1.609544641039</x:v>
       </x:c>
       <x:c r="G83" s="42" t="str">
-        <x:v>40.366162616318</x:v>
+        <x:v>1.609544641039</x:v>
       </x:c>
       <x:c r="H83" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3638,19 +3638,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C84" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D84" s="42" t="str">
-        <x:v>-21.728016057439</x:v>
+        <x:v>-40.056162616318</x:v>
       </x:c>
       <x:c r="E84" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F84" s="42" t="str">
-        <x:v>-22.978016057439</x:v>
+        <x:v>-40.366162616318</x:v>
       </x:c>
       <x:c r="G84" s="42" t="str">
-        <x:v>22.978016057439</x:v>
+        <x:v>40.366162616318</x:v>
       </x:c>
       <x:c r="H84" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3664,19 +3664,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C85" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D85" s="42" t="str">
-        <x:v>14.909575775296</x:v>
+        <x:v>-21.728016057439</x:v>
       </x:c>
       <x:c r="E85" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F85" s="42" t="str">
-        <x:v>11.079575775296</x:v>
+        <x:v>-22.978016057439</x:v>
       </x:c>
       <x:c r="G85" s="42" t="str">
-        <x:v>11.079575775296</x:v>
+        <x:v>22.978016057439</x:v>
       </x:c>
       <x:c r="H85" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3690,19 +3690,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C86" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D86" s="42" t="str">
-        <x:v>-57.502753280215</x:v>
+        <x:v>14.909575775296</x:v>
       </x:c>
       <x:c r="E86" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F86" s="42" t="str">
-        <x:v>-59.282753280215</x:v>
+        <x:v>11.079575775296</x:v>
       </x:c>
       <x:c r="G86" s="42" t="str">
-        <x:v>59.282753280215</x:v>
+        <x:v>11.079575775296</x:v>
       </x:c>
       <x:c r="H86" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3716,19 +3716,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C87" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D87" s="42" t="str">
-        <x:v>-300.067320161804</x:v>
+        <x:v>-57.502753280215</x:v>
       </x:c>
       <x:c r="E87" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F87" s="42" t="str">
-        <x:v>-305.057320161804</x:v>
+        <x:v>-59.282753280215</x:v>
       </x:c>
       <x:c r="G87" s="42" t="str">
-        <x:v>305.057320161804</x:v>
+        <x:v>59.282753280215</x:v>
       </x:c>
       <x:c r="H87" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3742,19 +3742,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C88" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D88" s="42" t="str">
-        <x:v>-121.498882525679</x:v>
+        <x:v>-300.067320161804</x:v>
       </x:c>
       <x:c r="E88" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F88" s="42" t="str">
-        <x:v>-125.728882525679</x:v>
+        <x:v>-305.057320161804</x:v>
       </x:c>
       <x:c r="G88" s="42" t="str">
-        <x:v>125.728882525679</x:v>
+        <x:v>305.057320161804</x:v>
       </x:c>
       <x:c r="H88" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3768,19 +3768,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C89" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D89" s="42" t="str">
-        <x:v>-14.812836787859</x:v>
+        <x:v>-121.498882525679</x:v>
       </x:c>
       <x:c r="E89" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F89" s="42" t="str">
-        <x:v>-15.412836787859</x:v>
+        <x:v>-125.728882525679</x:v>
       </x:c>
       <x:c r="G89" s="42" t="str">
-        <x:v>15.412836787859</x:v>
+        <x:v>125.728882525679</x:v>
       </x:c>
       <x:c r="H89" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3794,19 +3794,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C90" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D90" s="42" t="str">
-        <x:v>-165.257377908596</x:v>
+        <x:v>-14.812836787859</x:v>
       </x:c>
       <x:c r="E90" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F90" s="42" t="str">
-        <x:v>-165.417377908596</x:v>
+        <x:v>-15.412836787859</x:v>
       </x:c>
       <x:c r="G90" s="42" t="str">
-        <x:v>165.417377908596</x:v>
+        <x:v>15.412836787859</x:v>
       </x:c>
       <x:c r="H90" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3820,19 +3820,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C91" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D91" s="42" t="str">
-        <x:v>6.868364020212</x:v>
+        <x:v>-165.257377908596</x:v>
       </x:c>
       <x:c r="E91" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F91" s="42" t="str">
-        <x:v>4.748364020212</x:v>
+        <x:v>-165.417377908596</x:v>
       </x:c>
       <x:c r="G91" s="42" t="str">
-        <x:v>4.748364020212</x:v>
+        <x:v>165.417377908596</x:v>
       </x:c>
       <x:c r="H91" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3846,19 +3846,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C92" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D92" s="42" t="str">
-        <x:v>-199.611684777200</x:v>
+        <x:v>6.868364020212</x:v>
       </x:c>
       <x:c r="E92" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F92" s="42" t="str">
-        <x:v>-201.311684777200</x:v>
+        <x:v>4.748364020212</x:v>
       </x:c>
       <x:c r="G92" s="42" t="str">
-        <x:v>201.311684777200</x:v>
+        <x:v>4.748364020212</x:v>
       </x:c>
       <x:c r="H92" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3872,19 +3872,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C93" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D93" s="42" t="str">
-        <x:v>-58.050293332028</x:v>
+        <x:v>-199.611684777200</x:v>
       </x:c>
       <x:c r="E93" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F93" s="42" t="str">
-        <x:v>-59.790293332028</x:v>
+        <x:v>-201.311684777200</x:v>
       </x:c>
       <x:c r="G93" s="42" t="str">
-        <x:v>59.790293332028</x:v>
+        <x:v>201.311684777200</x:v>
       </x:c>
       <x:c r="H93" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3898,19 +3898,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C94" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D94" s="42" t="str">
-        <x:v>-51.559121420866</x:v>
+        <x:v>-58.050293332028</x:v>
       </x:c>
       <x:c r="E94" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F94" s="42" t="str">
-        <x:v>-53.309121420866</x:v>
+        <x:v>-59.790293332028</x:v>
       </x:c>
       <x:c r="G94" s="42" t="str">
-        <x:v>53.309121420866</x:v>
+        <x:v>59.790293332028</x:v>
       </x:c>
       <x:c r="H94" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3921,22 +3921,22 @@
         <x:v>author pbc CLI</x:v>
       </x:c>
       <x:c r="B95" s="36" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C95" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D95" s="42" t="str">
-        <x:v>-9.054674468559</x:v>
+        <x:v>-51.559121420866</x:v>
       </x:c>
       <x:c r="E95" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F95" s="42" t="str">
-        <x:v>-9.364674468559</x:v>
+        <x:v>-53.309121420866</x:v>
       </x:c>
       <x:c r="G95" s="42" t="str">
-        <x:v>9.364674468559</x:v>
+        <x:v>53.309121420866</x:v>
       </x:c>
       <x:c r="H95" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3950,19 +3950,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C96" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D96" s="42" t="str">
-        <x:v>-2.341718734421</x:v>
+        <x:v>-9.054674468559</x:v>
       </x:c>
       <x:c r="E96" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F96" s="42" t="str">
-        <x:v>-3.591718734421</x:v>
+        <x:v>-9.364674468559</x:v>
       </x:c>
       <x:c r="G96" s="42" t="str">
-        <x:v>3.591718734421</x:v>
+        <x:v>9.364674468559</x:v>
       </x:c>
       <x:c r="H96" s="36" t="str">
         <x:v>PASS</x:v>
@@ -3976,19 +3976,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C97" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D97" s="42" t="str">
-        <x:v>2.892295286943</x:v>
+        <x:v>-2.341718734421</x:v>
       </x:c>
       <x:c r="E97" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F97" s="42" t="str">
-        <x:v>-0.937704713057</x:v>
+        <x:v>-3.591718734421</x:v>
       </x:c>
       <x:c r="G97" s="42" t="str">
-        <x:v>0.937704713057</x:v>
+        <x:v>3.591718734421</x:v>
       </x:c>
       <x:c r="H97" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4002,19 +4002,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C98" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D98" s="42" t="str">
-        <x:v>-12.421511801622</x:v>
+        <x:v>2.892295286943</x:v>
       </x:c>
       <x:c r="E98" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F98" s="42" t="str">
-        <x:v>-14.201511801622</x:v>
+        <x:v>-0.937704713057</x:v>
       </x:c>
       <x:c r="G98" s="42" t="str">
-        <x:v>14.201511801622</x:v>
+        <x:v>0.937704713057</x:v>
       </x:c>
       <x:c r="H98" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4028,19 +4028,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C99" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D99" s="42" t="str">
-        <x:v>-153.975297576434</x:v>
+        <x:v>-12.421511801622</x:v>
       </x:c>
       <x:c r="E99" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F99" s="42" t="str">
-        <x:v>-158.965297576434</x:v>
+        <x:v>-14.201511801622</x:v>
       </x:c>
       <x:c r="G99" s="42" t="str">
-        <x:v>158.965297576434</x:v>
+        <x:v>14.201511801622</x:v>
       </x:c>
       <x:c r="H99" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4054,19 +4054,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C100" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D100" s="42" t="str">
-        <x:v>-38.490190110106</x:v>
+        <x:v>-153.975297576434</x:v>
       </x:c>
       <x:c r="E100" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F100" s="42" t="str">
-        <x:v>-42.720190110106</x:v>
+        <x:v>-158.965297576434</x:v>
       </x:c>
       <x:c r="G100" s="42" t="str">
-        <x:v>42.720190110106</x:v>
+        <x:v>158.965297576434</x:v>
       </x:c>
       <x:c r="H100" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4080,19 +4080,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C101" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D101" s="42" t="str">
-        <x:v>-2.462552657305</x:v>
+        <x:v>-38.490190110106</x:v>
       </x:c>
       <x:c r="E101" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F101" s="42" t="str">
-        <x:v>-3.062552657305</x:v>
+        <x:v>-42.720190110106</x:v>
       </x:c>
       <x:c r="G101" s="42" t="str">
-        <x:v>3.062552657305</x:v>
+        <x:v>42.720190110106</x:v>
       </x:c>
       <x:c r="H101" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4106,19 +4106,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C102" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D102" s="42" t="str">
-        <x:v>-62.538655042867</x:v>
+        <x:v>-2.462552657305</x:v>
       </x:c>
       <x:c r="E102" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F102" s="42" t="str">
-        <x:v>-62.698655042867</x:v>
+        <x:v>-3.062552657305</x:v>
       </x:c>
       <x:c r="G102" s="42" t="str">
-        <x:v>62.698655042867</x:v>
+        <x:v>3.062552657305</x:v>
       </x:c>
       <x:c r="H102" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4132,19 +4132,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C103" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D103" s="42" t="str">
-        <x:v>0.923689537732</x:v>
+        <x:v>-62.538655042867</x:v>
       </x:c>
       <x:c r="E103" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F103" s="42" t="str">
-        <x:v>-1.196310462268</x:v>
+        <x:v>-62.698655042867</x:v>
       </x:c>
       <x:c r="G103" s="42" t="str">
-        <x:v>1.196310462268</x:v>
+        <x:v>62.698655042867</x:v>
       </x:c>
       <x:c r="H103" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4158,19 +4158,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C104" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D104" s="42" t="str">
-        <x:v>-83.903026598902</x:v>
+        <x:v>0.923689537732</x:v>
       </x:c>
       <x:c r="E104" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F104" s="42" t="str">
-        <x:v>-85.603026598902</x:v>
+        <x:v>-1.196310462268</x:v>
       </x:c>
       <x:c r="G104" s="42" t="str">
-        <x:v>85.603026598902</x:v>
+        <x:v>1.196310462268</x:v>
       </x:c>
       <x:c r="H104" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4184,19 +4184,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C105" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D105" s="42" t="str">
-        <x:v>-12.548998010281</x:v>
+        <x:v>-83.903026598902</x:v>
       </x:c>
       <x:c r="E105" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F105" s="42" t="str">
-        <x:v>-14.288998010281</x:v>
+        <x:v>-85.603026598902</x:v>
       </x:c>
       <x:c r="G105" s="42" t="str">
-        <x:v>14.288998010281</x:v>
+        <x:v>85.603026598902</x:v>
       </x:c>
       <x:c r="H105" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4210,19 +4210,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C106" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D106" s="42" t="str">
-        <x:v>-10.466416914384</x:v>
+        <x:v>-12.548998010281</x:v>
       </x:c>
       <x:c r="E106" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F106" s="42" t="str">
-        <x:v>-12.216416914384</x:v>
+        <x:v>-14.288998010281</x:v>
       </x:c>
       <x:c r="G106" s="42" t="str">
-        <x:v>12.216416914384</x:v>
+        <x:v>14.288998010281</x:v>
       </x:c>
       <x:c r="H106" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4230,25 +4230,25 @@
     </x:row>
     <x:row r="107" ht="15" hidden="0" customHeight="1">
       <x:c r="A107" s="36" t="str">
-        <x:v>current pbc CLI</x:v>
+        <x:v>author pbc CLI</x:v>
       </x:c>
       <x:c r="B107" s="36" t="str">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C107" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D107" s="42" t="str">
-        <x:v>-85.402832480791</x:v>
+        <x:v>-10.466416914384</x:v>
       </x:c>
       <x:c r="E107" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F107" s="42" t="str">
-        <x:v>-85.712832480791</x:v>
+        <x:v>-12.216416914384</x:v>
       </x:c>
       <x:c r="G107" s="42" t="str">
-        <x:v>85.712832480791</x:v>
+        <x:v>12.216416914384</x:v>
       </x:c>
       <x:c r="H107" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4262,19 +4262,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C108" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D108" s="42" t="str">
-        <x:v>-52.784771448006</x:v>
+        <x:v>-85.402832480791</x:v>
       </x:c>
       <x:c r="E108" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F108" s="42" t="str">
-        <x:v>-54.034771448006</x:v>
+        <x:v>-85.712832480791</x:v>
       </x:c>
       <x:c r="G108" s="42" t="str">
-        <x:v>54.034771448006</x:v>
+        <x:v>85.712832480791</x:v>
       </x:c>
       <x:c r="H108" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4288,19 +4288,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C109" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D109" s="42" t="str">
-        <x:v>38.666296487481</x:v>
+        <x:v>-52.784771448006</x:v>
       </x:c>
       <x:c r="E109" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F109" s="42" t="str">
-        <x:v>34.836296487481</x:v>
+        <x:v>-54.034771448006</x:v>
       </x:c>
       <x:c r="G109" s="42" t="str">
-        <x:v>34.836296487481</x:v>
+        <x:v>54.034771448006</x:v>
       </x:c>
       <x:c r="H109" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4314,19 +4314,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C110" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D110" s="42" t="str">
-        <x:v>-119.951876462899</x:v>
+        <x:v>38.666296487481</x:v>
       </x:c>
       <x:c r="E110" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F110" s="42" t="str">
-        <x:v>-121.731876462899</x:v>
+        <x:v>34.836296487481</x:v>
       </x:c>
       <x:c r="G110" s="42" t="str">
-        <x:v>121.731876462899</x:v>
+        <x:v>34.836296487481</x:v>
       </x:c>
       <x:c r="H110" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4340,19 +4340,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C111" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D111" s="42" t="str">
-        <x:v>-491.873083815613</x:v>
+        <x:v>-119.951876462899</x:v>
       </x:c>
       <x:c r="E111" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F111" s="42" t="str">
-        <x:v>-496.863083815613</x:v>
+        <x:v>-121.731876462899</x:v>
       </x:c>
       <x:c r="G111" s="42" t="str">
-        <x:v>496.863083815613</x:v>
+        <x:v>121.731876462899</x:v>
       </x:c>
       <x:c r="H111" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4366,19 +4366,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C112" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D112" s="42" t="str">
-        <x:v>-227.181421040355</x:v>
+        <x:v>-491.873083815613</x:v>
       </x:c>
       <x:c r="E112" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F112" s="42" t="str">
-        <x:v>-231.411421040355</x:v>
+        <x:v>-496.863083815613</x:v>
       </x:c>
       <x:c r="G112" s="42" t="str">
-        <x:v>231.411421040355</x:v>
+        <x:v>496.863083815613</x:v>
       </x:c>
       <x:c r="H112" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4392,19 +4392,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C113" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D113" s="42" t="str">
-        <x:v>-36.269951925783</x:v>
+        <x:v>-227.181421040355</x:v>
       </x:c>
       <x:c r="E113" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F113" s="42" t="str">
-        <x:v>-36.869951925783</x:v>
+        <x:v>-231.411421040355</x:v>
       </x:c>
       <x:c r="G113" s="42" t="str">
-        <x:v>36.869951925783</x:v>
+        <x:v>231.411421040355</x:v>
       </x:c>
       <x:c r="H113" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4418,19 +4418,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C114" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D114" s="42" t="str">
-        <x:v>-299.258518836626</x:v>
+        <x:v>-36.269951925783</x:v>
       </x:c>
       <x:c r="E114" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F114" s="42" t="str">
-        <x:v>-299.418518836626</x:v>
+        <x:v>-36.869951925783</x:v>
       </x:c>
       <x:c r="G114" s="42" t="str">
-        <x:v>299.418518836626</x:v>
+        <x:v>36.869951925783</x:v>
       </x:c>
       <x:c r="H114" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4444,19 +4444,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C115" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D115" s="42" t="str">
-        <x:v>16.464730608559</x:v>
+        <x:v>-299.258518836626</x:v>
       </x:c>
       <x:c r="E115" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F115" s="42" t="str">
-        <x:v>14.344730608559</x:v>
+        <x:v>-299.418518836626</x:v>
       </x:c>
       <x:c r="G115" s="42" t="str">
-        <x:v>14.344730608559</x:v>
+        <x:v>299.418518836626</x:v>
       </x:c>
       <x:c r="H115" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4470,19 +4470,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C116" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D116" s="42" t="str">
-        <x:v>-351.956576532881</x:v>
+        <x:v>16.464730608559</x:v>
       </x:c>
       <x:c r="E116" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F116" s="42" t="str">
-        <x:v>-353.656576532881</x:v>
+        <x:v>14.344730608559</x:v>
       </x:c>
       <x:c r="G116" s="42" t="str">
-        <x:v>353.656576532881</x:v>
+        <x:v>14.344730608559</x:v>
       </x:c>
       <x:c r="H116" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4496,19 +4496,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C117" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D117" s="42" t="str">
-        <x:v>-121.156628176656</x:v>
+        <x:v>-351.956576532881</x:v>
       </x:c>
       <x:c r="E117" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F117" s="42" t="str">
-        <x:v>-122.896628176656</x:v>
+        <x:v>-353.656576532881</x:v>
       </x:c>
       <x:c r="G117" s="42" t="str">
-        <x:v>122.896628176656</x:v>
+        <x:v>353.656576532881</x:v>
       </x:c>
       <x:c r="H117" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4522,19 +4522,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C118" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D118" s="42" t="str">
-        <x:v>-112.486904450047</x:v>
+        <x:v>-121.156628176656</x:v>
       </x:c>
       <x:c r="E118" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F118" s="42" t="str">
-        <x:v>-114.236904450047</x:v>
+        <x:v>-122.896628176656</x:v>
       </x:c>
       <x:c r="G118" s="42" t="str">
-        <x:v>114.236904450047</x:v>
+        <x:v>122.896628176656</x:v>
       </x:c>
       <x:c r="H118" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4545,22 +4545,22 @@
         <x:v>current pbc CLI</x:v>
       </x:c>
       <x:c r="B119" s="36" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C119" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D119" s="42" t="str">
-        <x:v>-40.052769548562</x:v>
+        <x:v>-112.486904450047</x:v>
       </x:c>
       <x:c r="E119" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F119" s="42" t="str">
-        <x:v>-40.362769548562</x:v>
+        <x:v>-114.236904450047</x:v>
       </x:c>
       <x:c r="G119" s="42" t="str">
-        <x:v>40.362769548562</x:v>
+        <x:v>114.236904450047</x:v>
       </x:c>
       <x:c r="H119" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4574,19 +4574,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C120" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D120" s="42" t="str">
-        <x:v>-21.669458368756</x:v>
+        <x:v>-40.052769548562</x:v>
       </x:c>
       <x:c r="E120" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F120" s="42" t="str">
-        <x:v>-22.919458368756</x:v>
+        <x:v>-40.362769548562</x:v>
       </x:c>
       <x:c r="G120" s="42" t="str">
-        <x:v>22.919458368756</x:v>
+        <x:v>40.362769548562</x:v>
       </x:c>
       <x:c r="H120" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4600,19 +4600,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C121" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D121" s="42" t="str">
-        <x:v>14.926647908813</x:v>
+        <x:v>-21.669458368756</x:v>
       </x:c>
       <x:c r="E121" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F121" s="42" t="str">
-        <x:v>11.096647908813</x:v>
+        <x:v>-22.919458368756</x:v>
       </x:c>
       <x:c r="G121" s="42" t="str">
-        <x:v>11.096647908813</x:v>
+        <x:v>22.919458368756</x:v>
       </x:c>
       <x:c r="H121" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4626,19 +4626,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C122" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D122" s="42" t="str">
-        <x:v>-57.367276074495</x:v>
+        <x:v>14.926647908813</x:v>
       </x:c>
       <x:c r="E122" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F122" s="42" t="str">
-        <x:v>-59.147276074495</x:v>
+        <x:v>11.096647908813</x:v>
       </x:c>
       <x:c r="G122" s="42" t="str">
-        <x:v>59.147276074495</x:v>
+        <x:v>11.096647908813</x:v>
       </x:c>
       <x:c r="H122" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4652,19 +4652,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C123" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D123" s="42" t="str">
-        <x:v>-299.975204903283</x:v>
+        <x:v>-57.367276074495</x:v>
       </x:c>
       <x:c r="E123" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F123" s="42" t="str">
-        <x:v>-304.965204903283</x:v>
+        <x:v>-59.147276074495</x:v>
       </x:c>
       <x:c r="G123" s="42" t="str">
-        <x:v>304.965204903283</x:v>
+        <x:v>59.147276074495</x:v>
       </x:c>
       <x:c r="H123" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4678,19 +4678,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C124" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D124" s="42" t="str">
-        <x:v>-121.493623038083</x:v>
+        <x:v>-299.975204903283</x:v>
       </x:c>
       <x:c r="E124" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F124" s="42" t="str">
-        <x:v>-125.723623038083</x:v>
+        <x:v>-304.965204903283</x:v>
       </x:c>
       <x:c r="G124" s="42" t="str">
-        <x:v>125.723623038083</x:v>
+        <x:v>304.965204903283</x:v>
       </x:c>
       <x:c r="H124" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4704,19 +4704,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C125" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D125" s="42" t="str">
-        <x:v>-14.811033266160</x:v>
+        <x:v>-121.493623038083</x:v>
       </x:c>
       <x:c r="E125" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F125" s="42" t="str">
-        <x:v>-15.411033266160</x:v>
+        <x:v>-125.723623038083</x:v>
       </x:c>
       <x:c r="G125" s="42" t="str">
-        <x:v>15.411033266160</x:v>
+        <x:v>125.723623038083</x:v>
       </x:c>
       <x:c r="H125" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4730,19 +4730,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C126" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D126" s="42" t="str">
-        <x:v>-165.236809268426</x:v>
+        <x:v>-14.811033266160</x:v>
       </x:c>
       <x:c r="E126" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F126" s="42" t="str">
-        <x:v>-165.396809268426</x:v>
+        <x:v>-15.411033266160</x:v>
       </x:c>
       <x:c r="G126" s="42" t="str">
-        <x:v>165.396809268426</x:v>
+        <x:v>15.411033266160</x:v>
       </x:c>
       <x:c r="H126" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4756,19 +4756,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C127" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D127" s="42" t="str">
-        <x:v>6.872357662713</x:v>
+        <x:v>-165.236809268426</x:v>
       </x:c>
       <x:c r="E127" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F127" s="42" t="str">
-        <x:v>4.752357662713</x:v>
+        <x:v>-165.396809268426</x:v>
       </x:c>
       <x:c r="G127" s="42" t="str">
-        <x:v>4.752357662713</x:v>
+        <x:v>165.396809268426</x:v>
       </x:c>
       <x:c r="H127" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4782,19 +4782,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C128" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D128" s="42" t="str">
-        <x:v>-199.607041791688</x:v>
+        <x:v>6.872357662713</x:v>
       </x:c>
       <x:c r="E128" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F128" s="42" t="str">
-        <x:v>-201.307041791688</x:v>
+        <x:v>4.752357662713</x:v>
       </x:c>
       <x:c r="G128" s="42" t="str">
-        <x:v>201.307041791688</x:v>
+        <x:v>4.752357662713</x:v>
       </x:c>
       <x:c r="H128" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4808,19 +4808,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C129" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D129" s="42" t="str">
-        <x:v>-58.045564075785</x:v>
+        <x:v>-199.607041791688</x:v>
       </x:c>
       <x:c r="E129" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F129" s="42" t="str">
-        <x:v>-59.785564075785</x:v>
+        <x:v>-201.307041791688</x:v>
       </x:c>
       <x:c r="G129" s="42" t="str">
-        <x:v>59.785564075785</x:v>
+        <x:v>201.307041791688</x:v>
       </x:c>
       <x:c r="H129" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4834,19 +4834,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C130" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D130" s="42" t="str">
-        <x:v>-51.558720983607</x:v>
+        <x:v>-58.045564075785</x:v>
       </x:c>
       <x:c r="E130" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F130" s="42" t="str">
-        <x:v>-53.308720983607</x:v>
+        <x:v>-59.785564075785</x:v>
       </x:c>
       <x:c r="G130" s="42" t="str">
-        <x:v>53.308720983607</x:v>
+        <x:v>59.785564075785</x:v>
       </x:c>
       <x:c r="H130" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4857,22 +4857,22 @@
         <x:v>current pbc CLI</x:v>
       </x:c>
       <x:c r="B131" s="36" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C131" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D131" s="42" t="str">
-        <x:v>-9.052128552229</x:v>
+        <x:v>-51.558720983607</x:v>
       </x:c>
       <x:c r="E131" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F131" s="42" t="str">
-        <x:v>-9.362128552229</x:v>
+        <x:v>-53.308720983607</x:v>
       </x:c>
       <x:c r="G131" s="42" t="str">
-        <x:v>9.362128552229</x:v>
+        <x:v>53.308720983607</x:v>
       </x:c>
       <x:c r="H131" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4886,19 +4886,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C132" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D132" s="42" t="str">
-        <x:v>-2.299617048110</x:v>
+        <x:v>-9.052128552229</x:v>
       </x:c>
       <x:c r="E132" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F132" s="42" t="str">
-        <x:v>-3.549617048110</x:v>
+        <x:v>-9.362128552229</x:v>
       </x:c>
       <x:c r="G132" s="42" t="str">
-        <x:v>3.549617048110</x:v>
+        <x:v>9.362128552229</x:v>
       </x:c>
       <x:c r="H132" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4912,19 +4912,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C133" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D133" s="42" t="str">
-        <x:v>2.904340310370</x:v>
+        <x:v>-2.299617048110</x:v>
       </x:c>
       <x:c r="E133" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F133" s="42" t="str">
-        <x:v>-0.925659689630</x:v>
+        <x:v>-3.549617048110</x:v>
       </x:c>
       <x:c r="G133" s="42" t="str">
-        <x:v>0.925659689630</x:v>
+        <x:v>3.549617048110</x:v>
       </x:c>
       <x:c r="H133" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4938,19 +4938,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C134" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D134" s="42" t="str">
-        <x:v>-12.321031303355</x:v>
+        <x:v>2.904340310370</x:v>
       </x:c>
       <x:c r="E134" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F134" s="42" t="str">
-        <x:v>-14.101031303355</x:v>
+        <x:v>-0.925659689630</x:v>
       </x:c>
       <x:c r="G134" s="42" t="str">
-        <x:v>14.101031303355</x:v>
+        <x:v>0.925659689630</x:v>
       </x:c>
       <x:c r="H134" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4964,19 +4964,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C135" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D135" s="42" t="str">
-        <x:v>-153.898129900577</x:v>
+        <x:v>-12.321031303355</x:v>
       </x:c>
       <x:c r="E135" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F135" s="42" t="str">
-        <x:v>-158.888129900577</x:v>
+        <x:v>-14.101031303355</x:v>
       </x:c>
       <x:c r="G135" s="42" t="str">
-        <x:v>158.888129900577</x:v>
+        <x:v>14.101031303355</x:v>
       </x:c>
       <x:c r="H135" s="36" t="str">
         <x:v>PASS</x:v>
@@ -4990,19 +4990,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C136" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D136" s="42" t="str">
-        <x:v>-38.486266197120</x:v>
+        <x:v>-153.898129900577</x:v>
       </x:c>
       <x:c r="E136" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F136" s="42" t="str">
-        <x:v>-42.716266197120</x:v>
+        <x:v>-158.888129900577</x:v>
       </x:c>
       <x:c r="G136" s="42" t="str">
-        <x:v>42.716266197120</x:v>
+        <x:v>158.888129900577</x:v>
       </x:c>
       <x:c r="H136" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5016,19 +5016,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C137" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D137" s="42" t="str">
-        <x:v>-2.461004071112</x:v>
+        <x:v>-38.486266197120</x:v>
       </x:c>
       <x:c r="E137" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F137" s="42" t="str">
-        <x:v>-3.061004071112</x:v>
+        <x:v>-42.716266197120</x:v>
       </x:c>
       <x:c r="G137" s="42" t="str">
-        <x:v>3.061004071112</x:v>
+        <x:v>42.716266197120</x:v>
       </x:c>
       <x:c r="H137" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5042,19 +5042,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C138" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D138" s="42" t="str">
-        <x:v>-62.523175264048</x:v>
+        <x:v>-2.461004071112</x:v>
       </x:c>
       <x:c r="E138" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F138" s="42" t="str">
-        <x:v>-62.683175264048</x:v>
+        <x:v>-3.061004071112</x:v>
       </x:c>
       <x:c r="G138" s="42" t="str">
-        <x:v>62.683175264048</x:v>
+        <x:v>3.061004071112</x:v>
       </x:c>
       <x:c r="H138" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5068,19 +5068,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C139" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D139" s="42" t="str">
-        <x:v>0.926723486584</x:v>
+        <x:v>-62.523175264048</x:v>
       </x:c>
       <x:c r="E139" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F139" s="42" t="str">
-        <x:v>-1.193276513416</x:v>
+        <x:v>-62.683175264048</x:v>
       </x:c>
       <x:c r="G139" s="42" t="str">
-        <x:v>1.193276513416</x:v>
+        <x:v>62.683175264048</x:v>
       </x:c>
       <x:c r="H139" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5094,19 +5094,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C140" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D140" s="42" t="str">
-        <x:v>-83.899718986935</x:v>
+        <x:v>0.926723486584</x:v>
       </x:c>
       <x:c r="E140" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F140" s="42" t="str">
-        <x:v>-85.599718986935</x:v>
+        <x:v>-1.193276513416</x:v>
       </x:c>
       <x:c r="G140" s="42" t="str">
-        <x:v>85.599718986935</x:v>
+        <x:v>1.193276513416</x:v>
       </x:c>
       <x:c r="H140" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5120,19 +5120,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C141" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D141" s="42" t="str">
-        <x:v>-12.545503073689</x:v>
+        <x:v>-83.899718986935</x:v>
       </x:c>
       <x:c r="E141" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F141" s="42" t="str">
-        <x:v>-14.285503073689</x:v>
+        <x:v>-85.599718986935</x:v>
       </x:c>
       <x:c r="G141" s="42" t="str">
-        <x:v>14.285503073689</x:v>
+        <x:v>85.599718986935</x:v>
       </x:c>
       <x:c r="H141" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5146,19 +5146,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C142" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D142" s="42" t="str">
-        <x:v>-10.466391957817</x:v>
+        <x:v>-12.545503073689</x:v>
       </x:c>
       <x:c r="E142" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F142" s="42" t="str">
-        <x:v>-12.216391957817</x:v>
+        <x:v>-14.285503073689</x:v>
       </x:c>
       <x:c r="G142" s="42" t="str">
-        <x:v>12.216391957817</x:v>
+        <x:v>14.285503073689</x:v>
       </x:c>
       <x:c r="H142" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5169,22 +5169,22 @@
         <x:v>current pbc CLI</x:v>
       </x:c>
       <x:c r="B143" s="36" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C143" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D143" s="42" t="str">
-        <x:v>-2.513150603252</x:v>
+        <x:v>-10.466391957817</x:v>
       </x:c>
       <x:c r="E143" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F143" s="42" t="str">
-        <x:v>-2.823150603252</x:v>
+        <x:v>-12.216391957817</x:v>
       </x:c>
       <x:c r="G143" s="42" t="str">
-        <x:v>2.823150603252</x:v>
+        <x:v>12.216391957817</x:v>
       </x:c>
       <x:c r="H143" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5198,19 +5198,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C144" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D144" s="42" t="str">
-        <x:v>1.264029937698</x:v>
+        <x:v>-2.513150603252</x:v>
       </x:c>
       <x:c r="E144" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F144" s="42" t="str">
-        <x:v>0.014029937698</x:v>
+        <x:v>-2.823150603252</x:v>
       </x:c>
       <x:c r="G144" s="42" t="str">
-        <x:v>0.014029937698</x:v>
+        <x:v>2.823150603252</x:v>
       </x:c>
       <x:c r="H144" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5224,19 +5224,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C145" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D145" s="42" t="str">
-        <x:v>1.405712159485</x:v>
+        <x:v>1.264029937698</x:v>
       </x:c>
       <x:c r="E145" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F145" s="42" t="str">
-        <x:v>-2.424287840515</x:v>
+        <x:v>0.014029937698</x:v>
       </x:c>
       <x:c r="G145" s="42" t="str">
-        <x:v>2.424287840515</x:v>
+        <x:v>0.014029937698</x:v>
       </x:c>
       <x:c r="H145" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5250,19 +5250,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C146" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D146" s="42" t="str">
-        <x:v>-1.048061577331</x:v>
+        <x:v>1.405712159485</x:v>
       </x:c>
       <x:c r="E146" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F146" s="42" t="str">
-        <x:v>-2.828061577331</x:v>
+        <x:v>-2.424287840515</x:v>
       </x:c>
       <x:c r="G146" s="42" t="str">
-        <x:v>2.828061577331</x:v>
+        <x:v>2.424287840515</x:v>
       </x:c>
       <x:c r="H146" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5276,19 +5276,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C147" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D147" s="42" t="str">
-        <x:v>-63.955235096392</x:v>
+        <x:v>-1.048061577331</x:v>
       </x:c>
       <x:c r="E147" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F147" s="42" t="str">
-        <x:v>-68.945235096392</x:v>
+        <x:v>-2.828061577331</x:v>
       </x:c>
       <x:c r="G147" s="42" t="str">
-        <x:v>68.945235096392</x:v>
+        <x:v>2.828061577331</x:v>
       </x:c>
       <x:c r="H147" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5302,19 +5302,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C148" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D148" s="42" t="str">
-        <x:v>-6.163484047291</x:v>
+        <x:v>-63.955235096392</x:v>
       </x:c>
       <x:c r="E148" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F148" s="42" t="str">
-        <x:v>-10.393484047291</x:v>
+        <x:v>-68.945235096392</x:v>
       </x:c>
       <x:c r="G148" s="42" t="str">
-        <x:v>10.393484047291</x:v>
+        <x:v>68.945235096392</x:v>
       </x:c>
       <x:c r="H148" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5328,19 +5328,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C149" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D149" s="42" t="str">
-        <x:v>-0.372876272237</x:v>
+        <x:v>-6.163484047291</x:v>
       </x:c>
       <x:c r="E149" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F149" s="42" t="str">
-        <x:v>-0.972876272237</x:v>
+        <x:v>-10.393484047291</x:v>
       </x:c>
       <x:c r="G149" s="42" t="str">
-        <x:v>0.972876272237</x:v>
+        <x:v>10.393484047291</x:v>
       </x:c>
       <x:c r="H149" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5354,19 +5354,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C150" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D150" s="42" t="str">
-        <x:v>-14.875013200229</x:v>
+        <x:v>-0.372876272237</x:v>
       </x:c>
       <x:c r="E150" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F150" s="42" t="str">
-        <x:v>-15.035013200229</x:v>
+        <x:v>-0.972876272237</x:v>
       </x:c>
       <x:c r="G150" s="42" t="str">
-        <x:v>15.035013200229</x:v>
+        <x:v>0.972876272237</x:v>
       </x:c>
       <x:c r="H150" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5380,19 +5380,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C151" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D151" s="42" t="str">
-        <x:v>0.123061371006</x:v>
+        <x:v>-14.875013200229</x:v>
       </x:c>
       <x:c r="E151" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F151" s="42" t="str">
-        <x:v>-1.996938628994</x:v>
+        <x:v>-15.035013200229</x:v>
       </x:c>
       <x:c r="G151" s="42" t="str">
-        <x:v>1.996938628994</x:v>
+        <x:v>15.035013200229</x:v>
       </x:c>
       <x:c r="H151" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5406,19 +5406,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C152" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D152" s="42" t="str">
-        <x:v>-23.938106879109</x:v>
+        <x:v>0.123061371006</x:v>
       </x:c>
       <x:c r="E152" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F152" s="42" t="str">
-        <x:v>-25.638106879109</x:v>
+        <x:v>-1.996938628994</x:v>
       </x:c>
       <x:c r="G152" s="42" t="str">
-        <x:v>25.638106879109</x:v>
+        <x:v>1.996938628994</x:v>
       </x:c>
       <x:c r="H152" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5432,19 +5432,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C153" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D153" s="42" t="str">
-        <x:v>-1.097393985422</x:v>
+        <x:v>-23.938106879109</x:v>
       </x:c>
       <x:c r="E153" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F153" s="42" t="str">
-        <x:v>-2.837393985422</x:v>
+        <x:v>-25.638106879109</x:v>
       </x:c>
       <x:c r="G153" s="42" t="str">
-        <x:v>2.837393985422</x:v>
+        <x:v>25.638106879109</x:v>
       </x:c>
       <x:c r="H153" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5458,19 +5458,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C154" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D154" s="42" t="str">
-        <x:v>-0.727230275074</x:v>
+        <x:v>-1.097393985422</x:v>
       </x:c>
       <x:c r="E154" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F154" s="42" t="str">
-        <x:v>-2.477230275074</x:v>
+        <x:v>-2.837393985422</x:v>
       </x:c>
       <x:c r="G154" s="42" t="str">
-        <x:v>2.477230275074</x:v>
+        <x:v>2.837393985422</x:v>
       </x:c>
       <x:c r="H154" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5478,25 +5478,25 @@
     </x:row>
     <x:row r="155" ht="15" hidden="0" customHeight="1">
       <x:c r="A155" s="36" t="str">
-        <x:v>historical mstore-inorganic CLI</x:v>
+        <x:v>current pbc CLI</x:v>
       </x:c>
       <x:c r="B155" s="36" t="str">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C155" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D155" s="42" t="str">
-        <x:v>21.964390394634</x:v>
+        <x:v>-0.727230275074</x:v>
       </x:c>
       <x:c r="E155" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F155" s="42" t="str">
-        <x:v>21.654390394634</x:v>
+        <x:v>-2.477230275074</x:v>
       </x:c>
       <x:c r="G155" s="42" t="str">
-        <x:v>21.654390394634</x:v>
+        <x:v>2.477230275074</x:v>
       </x:c>
       <x:c r="H155" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5510,19 +5510,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C156" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D156" s="42" t="str">
-        <x:v>-171.325848518761</x:v>
+        <x:v>21.964390394634</x:v>
       </x:c>
       <x:c r="E156" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F156" s="42" t="str">
-        <x:v>-172.575848518761</x:v>
+        <x:v>21.654390394634</x:v>
       </x:c>
       <x:c r="G156" s="42" t="str">
-        <x:v>172.575848518761</x:v>
+        <x:v>21.654390394634</x:v>
       </x:c>
       <x:c r="H156" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5536,19 +5536,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C157" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D157" s="42" t="str">
-        <x:v>-64.481456672543</x:v>
+        <x:v>-171.325848518761</x:v>
       </x:c>
       <x:c r="E157" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F157" s="42" t="str">
-        <x:v>-68.311456672543</x:v>
+        <x:v>-172.575848518761</x:v>
       </x:c>
       <x:c r="G157" s="42" t="str">
-        <x:v>68.311456672543</x:v>
+        <x:v>172.575848518761</x:v>
       </x:c>
       <x:c r="H157" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5562,19 +5562,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C158" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D158" s="42" t="str">
-        <x:v>-55.475838468692</x:v>
+        <x:v>-64.481456672543</x:v>
       </x:c>
       <x:c r="E158" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F158" s="42" t="str">
-        <x:v>-57.255838468692</x:v>
+        <x:v>-68.311456672543</x:v>
       </x:c>
       <x:c r="G158" s="42" t="str">
-        <x:v>57.255838468692</x:v>
+        <x:v>68.311456672543</x:v>
       </x:c>
       <x:c r="H158" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5588,19 +5588,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C159" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D159" s="42" t="str">
-        <x:v>-259.196245399110</x:v>
+        <x:v>-55.475838468692</x:v>
       </x:c>
       <x:c r="E159" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F159" s="42" t="str">
-        <x:v>-264.186245399110</x:v>
+        <x:v>-57.255838468692</x:v>
       </x:c>
       <x:c r="G159" s="42" t="str">
-        <x:v>264.186245399110</x:v>
+        <x:v>57.255838468692</x:v>
       </x:c>
       <x:c r="H159" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5614,19 +5614,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C160" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D160" s="42" t="str">
-        <x:v>-252.839445286494</x:v>
+        <x:v>-259.196245399110</x:v>
       </x:c>
       <x:c r="E160" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F160" s="42" t="str">
-        <x:v>-257.069445286494</x:v>
+        <x:v>-264.186245399110</x:v>
       </x:c>
       <x:c r="G160" s="42" t="str">
-        <x:v>257.069445286494</x:v>
+        <x:v>264.186245399110</x:v>
       </x:c>
       <x:c r="H160" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5640,19 +5640,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C161" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D161" s="42" t="str">
-        <x:v>-146.178117427308</x:v>
+        <x:v>-252.839445286494</x:v>
       </x:c>
       <x:c r="E161" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F161" s="42" t="str">
-        <x:v>-146.778117427308</x:v>
+        <x:v>-257.069445286494</x:v>
       </x:c>
       <x:c r="G161" s="42" t="str">
-        <x:v>146.778117427308</x:v>
+        <x:v>257.069445286494</x:v>
       </x:c>
       <x:c r="H161" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5666,19 +5666,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C162" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D162" s="42" t="str">
-        <x:v>-224.393887966522</x:v>
+        <x:v>-146.178117427308</x:v>
       </x:c>
       <x:c r="E162" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F162" s="42" t="str">
-        <x:v>-224.553887966522</x:v>
+        <x:v>-146.778117427308</x:v>
       </x:c>
       <x:c r="G162" s="42" t="str">
-        <x:v>224.553887966522</x:v>
+        <x:v>146.778117427308</x:v>
       </x:c>
       <x:c r="H162" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5692,19 +5692,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C163" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D163" s="42" t="str">
-        <x:v>-64.059726187434</x:v>
+        <x:v>-224.393887966522</x:v>
       </x:c>
       <x:c r="E163" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F163" s="42" t="str">
-        <x:v>-66.179726187434</x:v>
+        <x:v>-224.553887966522</x:v>
       </x:c>
       <x:c r="G163" s="42" t="str">
-        <x:v>66.179726187434</x:v>
+        <x:v>224.553887966522</x:v>
       </x:c>
       <x:c r="H163" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5718,19 +5718,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C164" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D164" s="42" t="str">
-        <x:v>-178.832658863162</x:v>
+        <x:v>-64.059726187434</x:v>
       </x:c>
       <x:c r="E164" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F164" s="42" t="str">
-        <x:v>-180.532658863162</x:v>
+        <x:v>-66.179726187434</x:v>
       </x:c>
       <x:c r="G164" s="42" t="str">
-        <x:v>180.532658863162</x:v>
+        <x:v>66.179726187434</x:v>
       </x:c>
       <x:c r="H164" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5744,19 +5744,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C165" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D165" s="42" t="str">
-        <x:v>-55.925167433801</x:v>
+        <x:v>-178.832658863162</x:v>
       </x:c>
       <x:c r="E165" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F165" s="42" t="str">
-        <x:v>-57.665167433801</x:v>
+        <x:v>-180.532658863162</x:v>
       </x:c>
       <x:c r="G165" s="42" t="str">
-        <x:v>57.665167433801</x:v>
+        <x:v>180.532658863162</x:v>
       </x:c>
       <x:c r="H165" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5770,19 +5770,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C166" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D166" s="42" t="str">
-        <x:v>-52.285059233270</x:v>
+        <x:v>-55.925167433801</x:v>
       </x:c>
       <x:c r="E166" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F166" s="42" t="str">
-        <x:v>-54.035059233270</x:v>
+        <x:v>-57.665167433801</x:v>
       </x:c>
       <x:c r="G166" s="42" t="str">
-        <x:v>54.035059233270</x:v>
+        <x:v>57.665167433801</x:v>
       </x:c>
       <x:c r="H166" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5793,22 +5793,22 @@
         <x:v>historical mstore-inorganic CLI</x:v>
       </x:c>
       <x:c r="B167" s="36" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C167" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D167" s="42" t="str">
-        <x:v>11.549596417487</x:v>
+        <x:v>-52.285059233270</x:v>
       </x:c>
       <x:c r="E167" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F167" s="42" t="str">
-        <x:v>11.239596417487</x:v>
+        <x:v>-54.035059233270</x:v>
       </x:c>
       <x:c r="G167" s="42" t="str">
-        <x:v>11.239596417487</x:v>
+        <x:v>54.035059233270</x:v>
       </x:c>
       <x:c r="H167" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5822,19 +5822,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C168" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D168" s="42" t="str">
-        <x:v>-29.811523391510</x:v>
+        <x:v>11.549596417487</x:v>
       </x:c>
       <x:c r="E168" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F168" s="42" t="str">
-        <x:v>-31.061523391510</x:v>
+        <x:v>11.239596417487</x:v>
       </x:c>
       <x:c r="G168" s="42" t="str">
-        <x:v>31.061523391510</x:v>
+        <x:v>11.239596417487</x:v>
       </x:c>
       <x:c r="H168" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5848,19 +5848,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C169" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D169" s="42" t="str">
-        <x:v>0.256599145141</x:v>
+        <x:v>-29.811523391510</x:v>
       </x:c>
       <x:c r="E169" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F169" s="42" t="str">
-        <x:v>-3.573400854859</x:v>
+        <x:v>-31.061523391510</x:v>
       </x:c>
       <x:c r="G169" s="42" t="str">
-        <x:v>3.573400854859</x:v>
+        <x:v>31.061523391510</x:v>
       </x:c>
       <x:c r="H169" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5874,19 +5874,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C170" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D170" s="42" t="str">
-        <x:v>-28.460677817350</x:v>
+        <x:v>0.256599145141</x:v>
       </x:c>
       <x:c r="E170" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F170" s="42" t="str">
-        <x:v>-30.240677817350</x:v>
+        <x:v>-3.573400854859</x:v>
       </x:c>
       <x:c r="G170" s="42" t="str">
-        <x:v>30.240677817350</x:v>
+        <x:v>3.573400854859</x:v>
       </x:c>
       <x:c r="H170" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5900,19 +5900,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C171" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D171" s="42" t="str">
-        <x:v>-151.947965741842</x:v>
+        <x:v>-28.460677817350</x:v>
       </x:c>
       <x:c r="E171" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F171" s="42" t="str">
-        <x:v>-156.937965741842</x:v>
+        <x:v>-30.240677817350</x:v>
       </x:c>
       <x:c r="G171" s="42" t="str">
-        <x:v>156.937965741842</x:v>
+        <x:v>30.240677817350</x:v>
       </x:c>
       <x:c r="H171" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5926,19 +5926,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C172" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D172" s="42" t="str">
-        <x:v>-77.417542603032</x:v>
+        <x:v>-151.947965741842</x:v>
       </x:c>
       <x:c r="E172" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F172" s="42" t="str">
-        <x:v>-81.647542603032</x:v>
+        <x:v>-156.937965741842</x:v>
       </x:c>
       <x:c r="G172" s="42" t="str">
-        <x:v>81.647542603032</x:v>
+        <x:v>156.937965741842</x:v>
       </x:c>
       <x:c r="H172" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5952,19 +5952,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C173" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D173" s="42" t="str">
-        <x:v>-24.470250890265</x:v>
+        <x:v>-77.417542603032</x:v>
       </x:c>
       <x:c r="E173" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F173" s="42" t="str">
-        <x:v>-25.070250890265</x:v>
+        <x:v>-81.647542603032</x:v>
       </x:c>
       <x:c r="G173" s="42" t="str">
-        <x:v>25.070250890265</x:v>
+        <x:v>81.647542603032</x:v>
       </x:c>
       <x:c r="H173" s="36" t="str">
         <x:v>PASS</x:v>
@@ -5978,19 +5978,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C174" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D174" s="42" t="str">
-        <x:v>-84.549975905731</x:v>
+        <x:v>-24.470250890265</x:v>
       </x:c>
       <x:c r="E174" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F174" s="42" t="str">
-        <x:v>-84.709975905731</x:v>
+        <x:v>-25.070250890265</x:v>
       </x:c>
       <x:c r="G174" s="42" t="str">
-        <x:v>84.709975905731</x:v>
+        <x:v>25.070250890265</x:v>
       </x:c>
       <x:c r="H174" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6004,19 +6004,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C175" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D175" s="42" t="str">
-        <x:v>0.922244833924</x:v>
+        <x:v>-84.549975905731</x:v>
       </x:c>
       <x:c r="E175" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F175" s="42" t="str">
-        <x:v>-1.197755166076</x:v>
+        <x:v>-84.709975905731</x:v>
       </x:c>
       <x:c r="G175" s="42" t="str">
-        <x:v>1.197755166076</x:v>
+        <x:v>84.709975905731</x:v>
       </x:c>
       <x:c r="H175" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6030,19 +6030,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C176" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D176" s="42" t="str">
-        <x:v>-99.557194036284</x:v>
+        <x:v>0.922244833924</x:v>
       </x:c>
       <x:c r="E176" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F176" s="42" t="str">
-        <x:v>-101.257194036284</x:v>
+        <x:v>-1.197755166076</x:v>
       </x:c>
       <x:c r="G176" s="42" t="str">
-        <x:v>101.257194036284</x:v>
+        <x:v>1.197755166076</x:v>
       </x:c>
       <x:c r="H176" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6056,19 +6056,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C177" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D177" s="42" t="str">
-        <x:v>-28.664951204286</x:v>
+        <x:v>-99.557194036284</x:v>
       </x:c>
       <x:c r="E177" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F177" s="42" t="str">
-        <x:v>-30.404951204286</x:v>
+        <x:v>-101.257194036284</x:v>
       </x:c>
       <x:c r="G177" s="42" t="str">
-        <x:v>30.404951204286</x:v>
+        <x:v>101.257194036284</x:v>
       </x:c>
       <x:c r="H177" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6082,19 +6082,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C178" s="36" t="str">
-        <x:v>XVII</x:v>
+        <x:v>XV</x:v>
       </x:c>
       <x:c r="D178" s="42" t="str">
-        <x:v>-25.438330429983</x:v>
+        <x:v>-28.664951204286</x:v>
       </x:c>
       <x:c r="E178" s="42" t="str">
-        <x:v>1.750000</x:v>
+        <x:v>1.740000</x:v>
       </x:c>
       <x:c r="F178" s="42" t="str">
-        <x:v>-27.188330429983</x:v>
+        <x:v>-30.404951204286</x:v>
       </x:c>
       <x:c r="G178" s="42" t="str">
-        <x:v>27.188330429983</x:v>
+        <x:v>30.404951204286</x:v>
       </x:c>
       <x:c r="H178" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6105,22 +6105,22 @@
         <x:v>historical mstore-inorganic CLI</x:v>
       </x:c>
       <x:c r="B179" s="36" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C179" s="36" t="str">
-        <x:v>II</x:v>
+        <x:v>XVII</x:v>
       </x:c>
       <x:c r="D179" s="42" t="str">
-        <x:v>-0.279988209907</x:v>
+        <x:v>-25.438330429983</x:v>
       </x:c>
       <x:c r="E179" s="42" t="str">
-        <x:v>0.310000</x:v>
+        <x:v>1.750000</x:v>
       </x:c>
       <x:c r="F179" s="42" t="str">
-        <x:v>-0.589988209907</x:v>
+        <x:v>-27.188330429983</x:v>
       </x:c>
       <x:c r="G179" s="42" t="str">
-        <x:v>0.589988209907</x:v>
+        <x:v>27.188330429983</x:v>
       </x:c>
       <x:c r="H179" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6134,19 +6134,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C180" s="36" t="str">
-        <x:v>III</x:v>
+        <x:v>II</x:v>
       </x:c>
       <x:c r="D180" s="42" t="str">
-        <x:v>-1.720202220170</x:v>
+        <x:v>-0.279988209907</x:v>
       </x:c>
       <x:c r="E180" s="42" t="str">
-        <x:v>1.250000</x:v>
+        <x:v>0.310000</x:v>
       </x:c>
       <x:c r="F180" s="42" t="str">
-        <x:v>-2.970202220170</x:v>
+        <x:v>-0.589988209907</x:v>
       </x:c>
       <x:c r="G180" s="42" t="str">
-        <x:v>2.970202220170</x:v>
+        <x:v>0.589988209907</x:v>
       </x:c>
       <x:c r="H180" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6160,19 +6160,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C181" s="36" t="str">
-        <x:v>IV</x:v>
+        <x:v>III</x:v>
       </x:c>
       <x:c r="D181" s="42" t="str">
-        <x:v>1.653583137544</x:v>
+        <x:v>-1.720202220170</x:v>
       </x:c>
       <x:c r="E181" s="42" t="str">
-        <x:v>3.830000</x:v>
+        <x:v>1.250000</x:v>
       </x:c>
       <x:c r="F181" s="42" t="str">
-        <x:v>-2.176416862456</x:v>
+        <x:v>-2.970202220170</x:v>
       </x:c>
       <x:c r="G181" s="42" t="str">
-        <x:v>2.176416862456</x:v>
+        <x:v>2.970202220170</x:v>
       </x:c>
       <x:c r="H181" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6186,19 +6186,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C182" s="36" t="str">
-        <x:v>VI</x:v>
+        <x:v>IV</x:v>
       </x:c>
       <x:c r="D182" s="42" t="str">
-        <x:v>-5.912105883998</x:v>
+        <x:v>1.653583137544</x:v>
       </x:c>
       <x:c r="E182" s="42" t="str">
-        <x:v>1.780000</x:v>
+        <x:v>3.830000</x:v>
       </x:c>
       <x:c r="F182" s="42" t="str">
-        <x:v>-7.692105883998</x:v>
+        <x:v>-2.176416862456</x:v>
       </x:c>
       <x:c r="G182" s="42" t="str">
-        <x:v>7.692105883998</x:v>
+        <x:v>2.176416862456</x:v>
       </x:c>
       <x:c r="H182" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6212,19 +6212,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C183" s="36" t="str">
-        <x:v>VII</x:v>
+        <x:v>VI</x:v>
       </x:c>
       <x:c r="D183" s="42" t="str">
-        <x:v>-77.446667006181</x:v>
+        <x:v>-5.912105883998</x:v>
       </x:c>
       <x:c r="E183" s="42" t="str">
-        <x:v>4.990000</x:v>
+        <x:v>1.780000</x:v>
       </x:c>
       <x:c r="F183" s="42" t="str">
-        <x:v>-82.436667006181</x:v>
+        <x:v>-7.692105883998</x:v>
       </x:c>
       <x:c r="G183" s="42" t="str">
-        <x:v>82.436667006181</x:v>
+        <x:v>7.692105883998</x:v>
       </x:c>
       <x:c r="H183" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6238,19 +6238,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C184" s="36" t="str">
-        <x:v>VIII</x:v>
+        <x:v>VII</x:v>
       </x:c>
       <x:c r="D184" s="42" t="str">
-        <x:v>-19.706722185486</x:v>
+        <x:v>-77.446667006181</x:v>
       </x:c>
       <x:c r="E184" s="42" t="str">
-        <x:v>4.230000</x:v>
+        <x:v>4.990000</x:v>
       </x:c>
       <x:c r="F184" s="42" t="str">
-        <x:v>-23.936722185486</x:v>
+        <x:v>-82.436667006181</x:v>
       </x:c>
       <x:c r="G184" s="42" t="str">
-        <x:v>23.936722185486</x:v>
+        <x:v>82.436667006181</x:v>
       </x:c>
       <x:c r="H184" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6264,19 +6264,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C185" s="36" t="str">
-        <x:v>IX</x:v>
+        <x:v>VIII</x:v>
       </x:c>
       <x:c r="D185" s="42" t="str">
-        <x:v>-2.774771626398</x:v>
+        <x:v>-19.706722185486</x:v>
       </x:c>
       <x:c r="E185" s="42" t="str">
-        <x:v>0.600000</x:v>
+        <x:v>4.230000</x:v>
       </x:c>
       <x:c r="F185" s="42" t="str">
-        <x:v>-3.374771626398</x:v>
+        <x:v>-23.936722185486</x:v>
       </x:c>
       <x:c r="G185" s="42" t="str">
-        <x:v>3.374771626398</x:v>
+        <x:v>23.936722185486</x:v>
       </x:c>
       <x:c r="H185" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6290,19 +6290,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C186" s="36" t="str">
-        <x:v>XI</x:v>
+        <x:v>IX</x:v>
       </x:c>
       <x:c r="D186" s="42" t="str">
-        <x:v>-31.168750655955</x:v>
+        <x:v>-2.774771626398</x:v>
       </x:c>
       <x:c r="E186" s="42" t="str">
-        <x:v>0.160000</x:v>
+        <x:v>0.600000</x:v>
       </x:c>
       <x:c r="F186" s="42" t="str">
-        <x:v>-31.328750655955</x:v>
+        <x:v>-3.374771626398</x:v>
       </x:c>
       <x:c r="G186" s="42" t="str">
-        <x:v>31.328750655955</x:v>
+        <x:v>3.374771626398</x:v>
       </x:c>
       <x:c r="H186" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6316,19 +6316,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C187" s="36" t="str">
-        <x:v>XIII</x:v>
+        <x:v>XI</x:v>
       </x:c>
       <x:c r="D187" s="42" t="str">
-        <x:v>0.442953962487</x:v>
+        <x:v>-31.168750655955</x:v>
       </x:c>
       <x:c r="E187" s="42" t="str">
-        <x:v>2.120000</x:v>
+        <x:v>0.160000</x:v>
       </x:c>
       <x:c r="F187" s="42" t="str">
-        <x:v>-1.677046037513</x:v>
+        <x:v>-31.328750655955</x:v>
       </x:c>
       <x:c r="G187" s="42" t="str">
-        <x:v>1.677046037513</x:v>
+        <x:v>31.328750655955</x:v>
       </x:c>
       <x:c r="H187" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6342,19 +6342,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C188" s="36" t="str">
-        <x:v>XIV</x:v>
+        <x:v>XIII</x:v>
       </x:c>
       <x:c r="D188" s="42" t="str">
-        <x:v>-41.779791859131</x:v>
+        <x:v>0.442953962487</x:v>
       </x:c>
       <x:c r="E188" s="42" t="str">
-        <x:v>1.700000</x:v>
+        <x:v>2.120000</x:v>
       </x:c>
       <x:c r="F188" s="42" t="str">
-        <x:v>-43.479791859131</x:v>
+        <x:v>-1.677046037513</x:v>
       </x:c>
       <x:c r="G188" s="42" t="str">
-        <x:v>43.479791859131</x:v>
+        <x:v>1.677046037513</x:v>
       </x:c>
       <x:c r="H188" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6368,19 +6368,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C189" s="36" t="str">
-        <x:v>XV</x:v>
+        <x:v>XIV</x:v>
       </x:c>
       <x:c r="D189" s="42" t="str">
-        <x:v>-5.934441749535</x:v>
+        <x:v>-41.779791859131</x:v>
       </x:c>
       <x:c r="E189" s="42" t="str">
-        <x:v>1.740000</x:v>
+        <x:v>1.700000</x:v>
       </x:c>
       <x:c r="F189" s="42" t="str">
-        <x:v>-7.674441749535</x:v>
+        <x:v>-43.479791859131</x:v>
       </x:c>
       <x:c r="G189" s="42" t="str">
-        <x:v>7.674441749535</x:v>
+        <x:v>43.479791859131</x:v>
       </x:c>
       <x:c r="H189" s="36" t="str">
         <x:v>PASS</x:v>
@@ -6394,21 +6394,47 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C190" s="36" t="str">
+        <x:v>XV</x:v>
+      </x:c>
+      <x:c r="D190" s="42" t="str">
+        <x:v>-5.934441749535</x:v>
+      </x:c>
+      <x:c r="E190" s="42" t="str">
+        <x:v>1.740000</x:v>
+      </x:c>
+      <x:c r="F190" s="42" t="str">
+        <x:v>-7.674441749535</x:v>
+      </x:c>
+      <x:c r="G190" s="42" t="str">
+        <x:v>7.674441749535</x:v>
+      </x:c>
+      <x:c r="H190" s="36" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="15" hidden="0" customHeight="1">
+      <x:c r="A191" s="36" t="str">
+        <x:v>historical mstore-inorganic CLI</x:v>
+      </x:c>
+      <x:c r="B191" s="36" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C191" s="36" t="str">
         <x:v>XVII</x:v>
       </x:c>
-      <x:c r="D190" s="42" t="str">
+      <x:c r="D191" s="42" t="str">
         <x:v>-4.880577524129</x:v>
       </x:c>
-      <x:c r="E190" s="42" t="str">
+      <x:c r="E191" s="42" t="str">
         <x:v>1.750000</x:v>
       </x:c>
-      <x:c r="F190" s="42" t="str">
+      <x:c r="F191" s="42" t="str">
         <x:v>-6.630577524129</x:v>
       </x:c>
-      <x:c r="G190" s="42" t="str">
+      <x:c r="G191" s="42" t="str">
         <x:v>6.630577524129</x:v>
       </x:c>
-      <x:c r="H190" s="36" t="str">
+      <x:c r="H191" s="36" t="str">
         <x:v>PASS</x:v>
       </x:c>
     </x:row>
@@ -11751,21 +11777,47 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="C82" s="36" t="str">
+        <x:v>XI</x:v>
+      </x:c>
+      <x:c r="D82" s="42" t="str">
+        <x:v>0.508805411655</x:v>
+      </x:c>
+      <x:c r="E82" s="42" t="str">
+        <x:v>0.160000</x:v>
+      </x:c>
+      <x:c r="F82" s="42" t="str">
+        <x:v>0.348805411655</x:v>
+      </x:c>
+      <x:c r="G82" s="42" t="str">
+        <x:v>0.348805411655</x:v>
+      </x:c>
+      <x:c r="H82" s="36" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="15" hidden="0" customHeight="1">
+      <x:c r="A83" s="36" t="str">
+        <x:v>CP2K-native pbc provider</x:v>
+      </x:c>
+      <x:c r="B83" s="36" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C83" s="36" t="str">
         <x:v>XIV</x:v>
       </x:c>
-      <x:c r="D82" s="42" t="str">
+      <x:c r="D83" s="42" t="str">
         <x:v>0.090455358961</x:v>
       </x:c>
-      <x:c r="E82" s="42" t="str">
+      <x:c r="E83" s="42" t="str">
         <x:v>1.700000</x:v>
       </x:c>
-      <x:c r="F82" s="42" t="str">
+      <x:c r="F83" s="42" t="str">
         <x:v>-1.609544641039</x:v>
       </x:c>
-      <x:c r="G82" s="42" t="str">
+      <x:c r="G83" s="42" t="str">
         <x:v>1.609544641039</x:v>
       </x:c>
-      <x:c r="H82" s="36" t="str">
+      <x:c r="H83" s="36" t="str">
         <x:v>PASS</x:v>
       </x:c>
     </x:row>

</xml_diff>